<commit_message>
Clean up, write to sheets
</commit_message>
<xml_diff>
--- a/intermediate/dashboard_output_lifeexpectancy.xlsx
+++ b/intermediate/dashboard_output_lifeexpectancy.xlsx
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="H7">
-        <v>0.8125</v>
+        <v>0.625</v>
       </c>
       <c r="I7">
         <v>2023</v>
@@ -752,7 +752,7 @@
         <v>2015</v>
       </c>
       <c r="O7">
-        <v>83.05000000000001</v>
+        <v>83.2</v>
       </c>
     </row>
     <row r="8">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="H12">
-        <v>1.625</v>
+        <v>1.5625</v>
       </c>
       <c r="I12">
         <v>2023</v>
@@ -1022,7 +1022,7 @@
         <v>2015</v>
       </c>
       <c r="O12">
-        <v>83.40000000000001</v>
+        <v>83.45</v>
       </c>
     </row>
     <row r="13">
@@ -1076,7 +1076,7 @@
         <v>2015</v>
       </c>
       <c r="O13">
-        <v>82.60000000000001</v>
+        <v>82.75</v>
       </c>
     </row>
     <row r="14">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="H14">
-        <v>1.3125</v>
+        <v>1.312500000000002</v>
       </c>
       <c r="I14">
         <v>2023</v>
@@ -1238,7 +1238,7 @@
         <v>2015</v>
       </c>
       <c r="O16">
-        <v>82.45</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="17">
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="H18">
-        <v>0.7062500000000007</v>
+        <v>0.7125000000000004</v>
       </c>
       <c r="I18">
         <v>2023</v>
@@ -1346,7 +1346,7 @@
         <v>2015</v>
       </c>
       <c r="O18">
-        <v>62.03999999999996</v>
+        <v>62.01999999999998</v>
       </c>
     </row>
     <row r="19">
@@ -1375,7 +1375,7 @@
         </is>
       </c>
       <c r="H19">
-        <v>2.625</v>
+        <v>2.625000000000002</v>
       </c>
       <c r="I19">
         <v>2023</v>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="H25">
-        <v>1.25</v>
+        <v>1.250000000000002</v>
       </c>
       <c r="I25">
         <v>2023</v>
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="H34">
-        <v>0.5625</v>
+        <v>0.4375</v>
       </c>
       <c r="I34">
         <v>2023</v>
@@ -2210,7 +2210,7 @@
         <v>2015</v>
       </c>
       <c r="O34">
-        <v>82.95</v>
+        <v>83.10000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -2318,7 +2318,7 @@
         <v>2015</v>
       </c>
       <c r="O36">
-        <v>82.80000000000001</v>
+        <v>82.95</v>
       </c>
     </row>
     <row r="37">
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="H39">
-        <v>1.081250000000002</v>
+        <v>1.087500000000002</v>
       </c>
       <c r="I39">
         <v>2023</v>
@@ -2480,7 +2480,7 @@
         <v>2015</v>
       </c>
       <c r="O39">
-        <v>61.63999999999997</v>
+        <v>61.61999999999998</v>
       </c>
     </row>
     <row r="40">
@@ -2563,7 +2563,7 @@
         </is>
       </c>
       <c r="H41">
-        <v>0.9812500000000011</v>
+        <v>0.9875000000000007</v>
       </c>
       <c r="I41">
         <v>2023</v>
@@ -2588,7 +2588,7 @@
         <v>2015</v>
       </c>
       <c r="O41">
-        <v>61.96000000000004</v>
+        <v>61.93999999999997</v>
       </c>
     </row>
     <row r="42">
@@ -3074,7 +3074,7 @@
         <v>2015</v>
       </c>
       <c r="O50">
-        <v>82.75</v>
+        <v>82.90000000000001</v>
       </c>
     </row>
     <row r="51">
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="H56">
-        <v>0.4375</v>
+        <v>0.4375000000000018</v>
       </c>
       <c r="I56">
         <v>2023</v>
@@ -3643,7 +3643,7 @@
         </is>
       </c>
       <c r="H61">
-        <v>1.375</v>
+        <v>1.3125</v>
       </c>
       <c r="I61">
         <v>2023</v>
@@ -3668,7 +3668,7 @@
         <v>2015</v>
       </c>
       <c r="O61">
-        <v>83.40000000000001</v>
+        <v>83.45</v>
       </c>
     </row>
     <row r="62">
@@ -3830,7 +3830,7 @@
         <v>2015</v>
       </c>
       <c r="O64">
-        <v>82.7</v>
+        <v>82.85000000000001</v>
       </c>
     </row>
     <row r="65">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H66">
-        <v>1.3125</v>
+        <v>1.125</v>
       </c>
       <c r="I66">
         <v>2023</v>
@@ -3938,7 +3938,7 @@
         <v>2015</v>
       </c>
       <c r="O66">
-        <v>83.05000000000001</v>
+        <v>83.2</v>
       </c>
     </row>
     <row r="67">
@@ -4154,7 +4154,7 @@
         <v>2015</v>
       </c>
       <c r="O70">
-        <v>82.45</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="71">
@@ -4183,7 +4183,7 @@
         </is>
       </c>
       <c r="H71">
-        <v>0.8125</v>
+        <v>0.8125000000000018</v>
       </c>
       <c r="I71">
         <v>2023</v>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="H74">
-        <v>0.8062500000000039</v>
+        <v>0.8125000000000036</v>
       </c>
       <c r="I74">
         <v>2023</v>
@@ -4370,7 +4370,7 @@
         <v>2015</v>
       </c>
       <c r="O74">
-        <v>61.31999999999999</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="75">
@@ -5342,7 +5342,7 @@
         <v>2015</v>
       </c>
       <c r="O92">
-        <v>82.75</v>
+        <v>82.90000000000001</v>
       </c>
     </row>
     <row r="93">
@@ -5479,7 +5479,7 @@
         </is>
       </c>
       <c r="H95">
-        <v>0.5</v>
+        <v>0.3125</v>
       </c>
       <c r="I95">
         <v>2023</v>
@@ -5504,7 +5504,7 @@
         <v>2015</v>
       </c>
       <c r="O95">
-        <v>83.10000000000001</v>
+        <v>83.25</v>
       </c>
     </row>
     <row r="96">
@@ -5558,7 +5558,7 @@
         <v>2015</v>
       </c>
       <c r="O96">
-        <v>83.15000000000001</v>
+        <v>83.30000000000001</v>
       </c>
     </row>
     <row r="97">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="H97">
-        <v>1.5</v>
+        <v>1.375</v>
       </c>
       <c r="I97">
         <v>2023</v>
@@ -5612,7 +5612,7 @@
         <v>2015</v>
       </c>
       <c r="O97">
-        <v>83.30000000000001</v>
+        <v>83.40000000000001</v>
       </c>
     </row>
     <row r="98">
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="H101">
-        <v>1.5</v>
+        <v>1.500000000000002</v>
       </c>
       <c r="I101">
         <v>2023</v>
@@ -6127,7 +6127,7 @@
         </is>
       </c>
       <c r="H107">
-        <v>2.25</v>
+        <v>2.125</v>
       </c>
       <c r="I107">
         <v>2023</v>
@@ -6152,7 +6152,7 @@
         <v>2015</v>
       </c>
       <c r="O107">
-        <v>83.30000000000001</v>
+        <v>83.40000000000001</v>
       </c>
     </row>
     <row r="108">
@@ -6746,7 +6746,7 @@
         <v>2015</v>
       </c>
       <c r="O118">
-        <v>82.65000000000001</v>
+        <v>82.80000000000001</v>
       </c>
     </row>
     <row r="119">
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="H122">
-        <v>1.5</v>
+        <v>1.500000000000002</v>
       </c>
       <c r="I122">
         <v>2023</v>
@@ -7369,7 +7369,7 @@
         </is>
       </c>
       <c r="H130">
-        <v>0.7125000000000039</v>
+        <v>0.7187500000000036</v>
       </c>
       <c r="I130">
         <v>2023</v>
@@ -7394,7 +7394,7 @@
         <v>2015</v>
       </c>
       <c r="O130">
-        <v>61.31999999999999</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="131">
@@ -7423,7 +7423,7 @@
         </is>
       </c>
       <c r="H131">
-        <v>0.875</v>
+        <v>0.8125</v>
       </c>
       <c r="I131">
         <v>2023</v>
@@ -7448,7 +7448,7 @@
         <v>2015</v>
       </c>
       <c r="O131">
-        <v>83.40000000000001</v>
+        <v>83.45</v>
       </c>
     </row>
     <row r="132">
@@ -7693,7 +7693,7 @@
         </is>
       </c>
       <c r="H136">
-        <v>1.512500000000001</v>
+        <v>1.518750000000001</v>
       </c>
       <c r="I136">
         <v>2023</v>
@@ -7718,7 +7718,7 @@
         <v>2015</v>
       </c>
       <c r="O136">
-        <v>61.96000000000004</v>
+        <v>61.93999999999997</v>
       </c>
     </row>
     <row r="137">
@@ -8071,7 +8071,7 @@
         </is>
       </c>
       <c r="H143">
-        <v>0.7375000000000007</v>
+        <v>0.7437500000000004</v>
       </c>
       <c r="I143">
         <v>2023</v>
@@ -8096,7 +8096,7 @@
         <v>2015</v>
       </c>
       <c r="O143">
-        <v>62.03999999999996</v>
+        <v>62.01999999999998</v>
       </c>
     </row>
     <row r="144">
@@ -8179,7 +8179,7 @@
         </is>
       </c>
       <c r="H145">
-        <v>1.25</v>
+        <v>1.250000000000002</v>
       </c>
       <c r="I145">
         <v>2023</v>
@@ -8258,7 +8258,7 @@
         <v>2015</v>
       </c>
       <c r="O146">
-        <v>82.75</v>
+        <v>82.90000000000001</v>
       </c>
     </row>
     <row r="147">
@@ -8287,7 +8287,7 @@
         </is>
       </c>
       <c r="H147">
-        <v>1.1875</v>
+        <v>1</v>
       </c>
       <c r="I147">
         <v>2023</v>
@@ -8312,7 +8312,7 @@
         <v>2015</v>
       </c>
       <c r="O147">
-        <v>83.15000000000001</v>
+        <v>83.30000000000001</v>
       </c>
     </row>
     <row r="148">
@@ -8474,7 +8474,7 @@
         <v>2015</v>
       </c>
       <c r="O150">
-        <v>82.80000000000001</v>
+        <v>82.95</v>
       </c>
     </row>
     <row r="151">
@@ -8989,7 +8989,7 @@
         </is>
       </c>
       <c r="H160">
-        <v>0.5</v>
+        <v>0.5000000000000018</v>
       </c>
       <c r="I160">
         <v>2023</v>
@@ -9068,7 +9068,7 @@
         <v>2015</v>
       </c>
       <c r="O161">
-        <v>82.65000000000001</v>
+        <v>82.80000000000001</v>
       </c>
     </row>
     <row r="162">
@@ -9151,7 +9151,7 @@
         </is>
       </c>
       <c r="H163">
-        <v>-5.249999999999982</v>
+        <v>-5.249999999999984</v>
       </c>
       <c r="I163">
         <v>2023</v>
@@ -9205,7 +9205,7 @@
         </is>
       </c>
       <c r="H164">
-        <v>2.1875</v>
+        <v>2</v>
       </c>
       <c r="I164">
         <v>2023</v>
@@ -9230,7 +9230,7 @@
         <v>2015</v>
       </c>
       <c r="O164">
-        <v>83.15000000000001</v>
+        <v>83.30000000000001</v>
       </c>
     </row>
     <row r="165">
@@ -9284,7 +9284,7 @@
         <v>2015</v>
       </c>
       <c r="O165">
-        <v>82.90000000000001</v>
+        <v>83.05000000000001</v>
       </c>
     </row>
     <row r="166">
@@ -9745,7 +9745,7 @@
         </is>
       </c>
       <c r="H174">
-        <v>1.750000000000012</v>
+        <v>1.756250000000012</v>
       </c>
       <c r="I174">
         <v>2023</v>
@@ -9770,7 +9770,7 @@
         <v>2015</v>
       </c>
       <c r="O174">
-        <v>59.40000000000001</v>
+        <v>59.37999999999993</v>
       </c>
     </row>
     <row r="175">
@@ -9932,7 +9932,7 @@
         <v>2015</v>
       </c>
       <c r="O177">
-        <v>59.07999999999993</v>
+        <v>59.05999999999995</v>
       </c>
     </row>
     <row r="178">
@@ -10015,7 +10015,7 @@
         </is>
       </c>
       <c r="H179">
-        <v>4.650000000000052</v>
+        <v>4.656250000000052</v>
       </c>
       <c r="I179">
         <v>2023</v>
@@ -10123,7 +10123,7 @@
         </is>
       </c>
       <c r="H181">
-        <v>1.875</v>
+        <v>1.875000000000002</v>
       </c>
       <c r="I181">
         <v>2023</v>
@@ -10285,7 +10285,7 @@
         </is>
       </c>
       <c r="H184">
-        <v>1.25</v>
+        <v>1.0625</v>
       </c>
       <c r="I184">
         <v>2023</v>
@@ -10310,7 +10310,7 @@
         <v>2015</v>
       </c>
       <c r="O184">
-        <v>83.10000000000001</v>
+        <v>83.25</v>
       </c>
     </row>
     <row r="185">
@@ -10339,7 +10339,7 @@
         </is>
       </c>
       <c r="H185">
-        <v>2.650000000000013</v>
+        <v>2.656250000000012</v>
       </c>
       <c r="I185">
         <v>2023</v>
@@ -10987,7 +10987,7 @@
         </is>
       </c>
       <c r="H197">
-        <v>0.375</v>
+        <v>0.3750000000000018</v>
       </c>
       <c r="I197">
         <v>2023</v>

</xml_diff>

<commit_message>
Life expectancy indicator, move meta_sheet.csv to input
</commit_message>
<xml_diff>
--- a/intermediate/dashboard_output_lifeexpectancy.xlsx
+++ b/intermediate/dashboard_output_lifeexpectancy.xlsx
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="H7">
-        <v>0.625</v>
+        <v>0.5625</v>
       </c>
       <c r="I7">
         <v>2023</v>
@@ -752,7 +752,7 @@
         <v>2015</v>
       </c>
       <c r="O7">
-        <v>83.2</v>
+        <v>83.25</v>
       </c>
     </row>
     <row r="8">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="H12">
-        <v>1.5625</v>
+        <v>1.5</v>
       </c>
       <c r="I12">
         <v>2023</v>
@@ -1022,7 +1022,7 @@
         <v>2015</v>
       </c>
       <c r="O12">
-        <v>83.45</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="13">
@@ -1076,7 +1076,7 @@
         <v>2015</v>
       </c>
       <c r="O13">
-        <v>82.75</v>
+        <v>82.80000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="H14">
-        <v>1.312500000000002</v>
+        <v>1.3125</v>
       </c>
       <c r="I14">
         <v>2023</v>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="H18">
-        <v>0.7125000000000004</v>
+        <v>0.71875</v>
       </c>
       <c r="I18">
         <v>2023</v>
@@ -1346,7 +1346,7 @@
         <v>2015</v>
       </c>
       <c r="O18">
-        <v>62.01999999999998</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19">
@@ -1375,7 +1375,7 @@
         </is>
       </c>
       <c r="H19">
-        <v>2.625000000000002</v>
+        <v>2.625</v>
       </c>
       <c r="I19">
         <v>2023</v>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="H25">
-        <v>1.250000000000002</v>
+        <v>1.25</v>
       </c>
       <c r="I25">
         <v>2023</v>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="H27">
-        <v>0.6666666666666607</v>
+        <v>0.6458333333333268</v>
       </c>
       <c r="I27">
         <v>2023</v>
@@ -1832,7 +1832,7 @@
         <v>2015</v>
       </c>
       <c r="O27">
-        <v>69.13333333333335</v>
+        <v>69.1666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="H32">
-        <v>2.645833333333307</v>
+        <v>2.624999999999973</v>
       </c>
       <c r="I32">
         <v>2023</v>
@@ -2210,7 +2210,7 @@
         <v>2015</v>
       </c>
       <c r="O34">
-        <v>83.10000000000001</v>
+        <v>83.15000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -2318,7 +2318,7 @@
         <v>2015</v>
       </c>
       <c r="O36">
-        <v>82.95</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37">
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="H39">
-        <v>1.087500000000002</v>
+        <v>1.093750000000002</v>
       </c>
       <c r="I39">
         <v>2023</v>
@@ -2480,7 +2480,7 @@
         <v>2015</v>
       </c>
       <c r="O39">
-        <v>61.61999999999998</v>
+        <v>61.6</v>
       </c>
     </row>
     <row r="40">
@@ -2563,7 +2563,7 @@
         </is>
       </c>
       <c r="H41">
-        <v>0.9875000000000007</v>
+        <v>0.9937500000000004</v>
       </c>
       <c r="I41">
         <v>2023</v>
@@ -2588,7 +2588,7 @@
         <v>2015</v>
       </c>
       <c r="O41">
-        <v>61.93999999999997</v>
+        <v>61.91999999999999</v>
       </c>
     </row>
     <row r="42">
@@ -3074,7 +3074,7 @@
         <v>2015</v>
       </c>
       <c r="O50">
-        <v>82.90000000000001</v>
+        <v>82.95</v>
       </c>
     </row>
     <row r="51">
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="H56">
-        <v>0.4375000000000018</v>
+        <v>0.4375</v>
       </c>
       <c r="I56">
         <v>2023</v>
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="H60">
-        <v>1.20833333333332</v>
+        <v>1.187499999999986</v>
       </c>
       <c r="I60">
         <v>2023</v>
@@ -3614,7 +3614,7 @@
         <v>2015</v>
       </c>
       <c r="O60">
-        <v>68.26666666666669</v>
+        <v>68.3</v>
       </c>
     </row>
     <row r="61">
@@ -3643,7 +3643,7 @@
         </is>
       </c>
       <c r="H61">
-        <v>1.3125</v>
+        <v>1.25</v>
       </c>
       <c r="I61">
         <v>2023</v>
@@ -3668,7 +3668,7 @@
         <v>2015</v>
       </c>
       <c r="O61">
-        <v>83.45</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="62">
@@ -3830,7 +3830,7 @@
         <v>2015</v>
       </c>
       <c r="O64">
-        <v>82.85000000000001</v>
+        <v>82.90000000000001</v>
       </c>
     </row>
     <row r="65">
@@ -3884,7 +3884,7 @@
         <v>2015</v>
       </c>
       <c r="O65">
-        <v>68.6666666666667</v>
+        <v>68.7</v>
       </c>
     </row>
     <row r="66">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H66">
-        <v>1.125</v>
+        <v>1.0625</v>
       </c>
       <c r="I66">
         <v>2023</v>
@@ -3938,7 +3938,7 @@
         <v>2015</v>
       </c>
       <c r="O66">
-        <v>83.2</v>
+        <v>83.25</v>
       </c>
     </row>
     <row r="67">
@@ -4075,7 +4075,7 @@
         </is>
       </c>
       <c r="H69">
-        <v>0.8541666666666554</v>
+        <v>0.8333333333333215</v>
       </c>
       <c r="I69">
         <v>2023</v>
@@ -4100,7 +4100,7 @@
         <v>2015</v>
       </c>
       <c r="O69">
-        <v>68.53333333333335</v>
+        <v>68.56666666666671</v>
       </c>
     </row>
     <row r="70">
@@ -4183,7 +4183,7 @@
         </is>
       </c>
       <c r="H71">
-        <v>0.8125000000000018</v>
+        <v>0.8125</v>
       </c>
       <c r="I71">
         <v>2023</v>
@@ -4291,7 +4291,7 @@
         </is>
       </c>
       <c r="H73">
-        <v>1.125</v>
+        <v>1.0625</v>
       </c>
       <c r="I73">
         <v>2023</v>
@@ -4316,7 +4316,7 @@
         <v>2015</v>
       </c>
       <c r="O73">
-        <v>83.5</v>
+        <v>83.55000000000001</v>
       </c>
     </row>
     <row r="74">
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="H74">
-        <v>0.8125000000000036</v>
+        <v>0.8187500000000032</v>
       </c>
       <c r="I74">
         <v>2023</v>
@@ -4370,7 +4370,7 @@
         <v>2015</v>
       </c>
       <c r="O74">
-        <v>61.3</v>
+        <v>61.28000000000002</v>
       </c>
     </row>
     <row r="75">
@@ -4831,7 +4831,7 @@
         </is>
       </c>
       <c r="H83">
-        <v>1.45833333333333</v>
+        <v>1.437499999999996</v>
       </c>
       <c r="I83">
         <v>2023</v>
@@ -4856,7 +4856,7 @@
         <v>2015</v>
       </c>
       <c r="O83">
-        <v>69.46666666666665</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="84">
@@ -5342,7 +5342,7 @@
         <v>2015</v>
       </c>
       <c r="O92">
-        <v>82.90000000000001</v>
+        <v>82.95</v>
       </c>
     </row>
     <row r="93">
@@ -5504,7 +5504,7 @@
         <v>2015</v>
       </c>
       <c r="O95">
-        <v>83.25</v>
+        <v>83.30000000000001</v>
       </c>
     </row>
     <row r="96">
@@ -5558,7 +5558,7 @@
         <v>2015</v>
       </c>
       <c r="O96">
-        <v>83.30000000000001</v>
+        <v>83.35000000000001</v>
       </c>
     </row>
     <row r="97">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="H97">
-        <v>1.375</v>
+        <v>1.3125</v>
       </c>
       <c r="I97">
         <v>2023</v>
@@ -5612,7 +5612,7 @@
         <v>2015</v>
       </c>
       <c r="O97">
-        <v>83.40000000000001</v>
+        <v>83.45</v>
       </c>
     </row>
     <row r="98">
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="H101">
-        <v>1.500000000000002</v>
+        <v>1.5</v>
       </c>
       <c r="I101">
         <v>2023</v>
@@ -6127,7 +6127,7 @@
         </is>
       </c>
       <c r="H107">
-        <v>2.125</v>
+        <v>2.0625</v>
       </c>
       <c r="I107">
         <v>2023</v>
@@ -6152,7 +6152,7 @@
         <v>2015</v>
       </c>
       <c r="O107">
-        <v>83.40000000000001</v>
+        <v>83.45</v>
       </c>
     </row>
     <row r="108">
@@ -6235,7 +6235,7 @@
         </is>
       </c>
       <c r="H109">
-        <v>1.124999999999991</v>
+        <v>1.104166666666657</v>
       </c>
       <c r="I109">
         <v>2023</v>
@@ -6260,7 +6260,7 @@
         <v>2015</v>
       </c>
       <c r="O109">
-        <v>68.8</v>
+        <v>68.83333333333334</v>
       </c>
     </row>
     <row r="110">
@@ -6746,7 +6746,7 @@
         <v>2015</v>
       </c>
       <c r="O118">
-        <v>82.80000000000001</v>
+        <v>82.85000000000001</v>
       </c>
     </row>
     <row r="119">
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="H122">
-        <v>1.500000000000002</v>
+        <v>1.5</v>
       </c>
       <c r="I122">
         <v>2023</v>
@@ -7369,7 +7369,7 @@
         </is>
       </c>
       <c r="H130">
-        <v>0.7187500000000036</v>
+        <v>0.7250000000000032</v>
       </c>
       <c r="I130">
         <v>2023</v>
@@ -7394,7 +7394,7 @@
         <v>2015</v>
       </c>
       <c r="O130">
-        <v>61.3</v>
+        <v>61.28000000000002</v>
       </c>
     </row>
     <row r="131">
@@ -7423,7 +7423,7 @@
         </is>
       </c>
       <c r="H131">
-        <v>0.8125</v>
+        <v>0.75</v>
       </c>
       <c r="I131">
         <v>2023</v>
@@ -7448,7 +7448,7 @@
         <v>2015</v>
       </c>
       <c r="O131">
-        <v>83.45</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="132">
@@ -7693,7 +7693,7 @@
         </is>
       </c>
       <c r="H136">
-        <v>1.518750000000001</v>
+        <v>1.525</v>
       </c>
       <c r="I136">
         <v>2023</v>
@@ -7718,7 +7718,7 @@
         <v>2015</v>
       </c>
       <c r="O136">
-        <v>61.93999999999997</v>
+        <v>61.91999999999999</v>
       </c>
     </row>
     <row r="137">
@@ -7747,7 +7747,7 @@
         </is>
       </c>
       <c r="H137">
-        <v>0.8958333333333233</v>
+        <v>0.8749999999999893</v>
       </c>
       <c r="I137">
         <v>2023</v>
@@ -7772,7 +7772,7 @@
         <v>2015</v>
       </c>
       <c r="O137">
-        <v>68.6666666666667</v>
+        <v>68.7</v>
       </c>
     </row>
     <row r="138">
@@ -8071,7 +8071,7 @@
         </is>
       </c>
       <c r="H143">
-        <v>0.7437500000000004</v>
+        <v>0.75</v>
       </c>
       <c r="I143">
         <v>2023</v>
@@ -8096,7 +8096,7 @@
         <v>2015</v>
       </c>
       <c r="O143">
-        <v>62.01999999999998</v>
+        <v>62</v>
       </c>
     </row>
     <row r="144">
@@ -8179,7 +8179,7 @@
         </is>
       </c>
       <c r="H145">
-        <v>1.250000000000002</v>
+        <v>1.25</v>
       </c>
       <c r="I145">
         <v>2023</v>
@@ -8258,7 +8258,7 @@
         <v>2015</v>
       </c>
       <c r="O146">
-        <v>82.90000000000001</v>
+        <v>82.95</v>
       </c>
     </row>
     <row r="147">
@@ -8287,7 +8287,7 @@
         </is>
       </c>
       <c r="H147">
-        <v>1</v>
+        <v>0.9375</v>
       </c>
       <c r="I147">
         <v>2023</v>
@@ -8312,7 +8312,7 @@
         <v>2015</v>
       </c>
       <c r="O147">
-        <v>83.30000000000001</v>
+        <v>83.35000000000001</v>
       </c>
     </row>
     <row r="148">
@@ -8341,7 +8341,7 @@
         </is>
       </c>
       <c r="H148">
-        <v>1.708333333333329</v>
+        <v>1.687499999999995</v>
       </c>
       <c r="I148">
         <v>2023</v>
@@ -8366,7 +8366,7 @@
         <v>2015</v>
       </c>
       <c r="O148">
-        <v>69.26666666666669</v>
+        <v>69.3</v>
       </c>
     </row>
     <row r="149">
@@ -8474,7 +8474,7 @@
         <v>2015</v>
       </c>
       <c r="O150">
-        <v>82.95</v>
+        <v>83</v>
       </c>
     </row>
     <row r="151">
@@ -8989,7 +8989,7 @@
         </is>
       </c>
       <c r="H160">
-        <v>0.5000000000000018</v>
+        <v>0.5</v>
       </c>
       <c r="I160">
         <v>2023</v>
@@ -9068,7 +9068,7 @@
         <v>2015</v>
       </c>
       <c r="O161">
-        <v>82.80000000000001</v>
+        <v>82.85000000000001</v>
       </c>
     </row>
     <row r="162">
@@ -9151,7 +9151,7 @@
         </is>
       </c>
       <c r="H163">
-        <v>-5.249999999999984</v>
+        <v>-5.229166666666648</v>
       </c>
       <c r="I163">
         <v>2023</v>
@@ -9205,7 +9205,7 @@
         </is>
       </c>
       <c r="H164">
-        <v>2</v>
+        <v>1.9375</v>
       </c>
       <c r="I164">
         <v>2023</v>
@@ -9230,7 +9230,7 @@
         <v>2015</v>
       </c>
       <c r="O164">
-        <v>83.30000000000001</v>
+        <v>83.35000000000001</v>
       </c>
     </row>
     <row r="165">
@@ -9284,7 +9284,7 @@
         <v>2015</v>
       </c>
       <c r="O165">
-        <v>83.05000000000001</v>
+        <v>83.10000000000001</v>
       </c>
     </row>
     <row r="166">
@@ -9583,7 +9583,7 @@
         </is>
       </c>
       <c r="H171">
-        <v>1.020833333333323</v>
+        <v>0.9999999999999893</v>
       </c>
       <c r="I171">
         <v>2023</v>
@@ -9608,7 +9608,7 @@
         <v>2015</v>
       </c>
       <c r="O171">
-        <v>68.6666666666667</v>
+        <v>68.7</v>
       </c>
     </row>
     <row r="172">
@@ -9637,7 +9637,7 @@
         </is>
       </c>
       <c r="H172">
-        <v>1.25</v>
+        <v>1.1875</v>
       </c>
       <c r="I172">
         <v>2023</v>
@@ -9662,7 +9662,7 @@
         <v>2015</v>
       </c>
       <c r="O172">
-        <v>83.5</v>
+        <v>83.55000000000001</v>
       </c>
     </row>
     <row r="173">
@@ -9745,7 +9745,7 @@
         </is>
       </c>
       <c r="H174">
-        <v>1.756250000000012</v>
+        <v>1.762500000000012</v>
       </c>
       <c r="I174">
         <v>2023</v>
@@ -9770,7 +9770,7 @@
         <v>2015</v>
       </c>
       <c r="O174">
-        <v>59.37999999999993</v>
+        <v>59.35999999999995</v>
       </c>
     </row>
     <row r="175">
@@ -9932,7 +9932,7 @@
         <v>2015</v>
       </c>
       <c r="O177">
-        <v>59.05999999999995</v>
+        <v>59.03999999999996</v>
       </c>
     </row>
     <row r="178">
@@ -10015,7 +10015,7 @@
         </is>
       </c>
       <c r="H179">
-        <v>4.656250000000052</v>
+        <v>4.650000000000052</v>
       </c>
       <c r="I179">
         <v>2023</v>
@@ -10069,7 +10069,7 @@
         </is>
       </c>
       <c r="H180">
-        <v>1.854166666666654</v>
+        <v>1.83333333333332</v>
       </c>
       <c r="I180">
         <v>2023</v>
@@ -10094,7 +10094,7 @@
         <v>2015</v>
       </c>
       <c r="O180">
-        <v>68.33333333333334</v>
+        <v>68.3666666666667</v>
       </c>
     </row>
     <row r="181">
@@ -10123,7 +10123,7 @@
         </is>
       </c>
       <c r="H181">
-        <v>1.875000000000002</v>
+        <v>1.875</v>
       </c>
       <c r="I181">
         <v>2023</v>
@@ -10285,7 +10285,7 @@
         </is>
       </c>
       <c r="H184">
-        <v>1.0625</v>
+        <v>1</v>
       </c>
       <c r="I184">
         <v>2023</v>
@@ -10310,7 +10310,7 @@
         <v>2015</v>
       </c>
       <c r="O184">
-        <v>83.25</v>
+        <v>83.30000000000001</v>
       </c>
     </row>
     <row r="185">
@@ -10339,7 +10339,7 @@
         </is>
       </c>
       <c r="H185">
-        <v>2.656250000000012</v>
+        <v>2.662500000000012</v>
       </c>
       <c r="I185">
         <v>2023</v>
@@ -10364,7 +10364,7 @@
         <v>2015</v>
       </c>
       <c r="O185">
-        <v>58.90000000000001</v>
+        <v>58.87999999999993</v>
       </c>
     </row>
     <row r="186">
@@ -10501,7 +10501,7 @@
         </is>
       </c>
       <c r="H188">
-        <v>4.427083333333307</v>
+        <v>4.406249999999973</v>
       </c>
       <c r="I188">
         <v>2023</v>
@@ -10987,7 +10987,7 @@
         </is>
       </c>
       <c r="H197">
-        <v>0.3750000000000018</v>
+        <v>0.375</v>
       </c>
       <c r="I197">
         <v>2023</v>
@@ -11311,7 +11311,7 @@
         </is>
       </c>
       <c r="H203">
-        <v>1.895833333333307</v>
+        <v>1.874999999999973</v>
       </c>
       <c r="I203">
         <v>2023</v>
@@ -12013,7 +12013,7 @@
         </is>
       </c>
       <c r="H216">
-        <v>1.270833333333325</v>
+        <v>1.249999999999991</v>
       </c>
       <c r="I216">
         <v>2023</v>
@@ -12038,7 +12038,7 @@
         <v>2015</v>
       </c>
       <c r="O216">
-        <v>68.8666666666667</v>
+        <v>68.90000000000001</v>
       </c>
     </row>
     <row r="217">

</xml_diff>

<commit_message>
Run scripts, add water
</commit_message>
<xml_diff>
--- a/intermediate/dashboard_output_lifeexpectancy.xlsx
+++ b/intermediate/dashboard_output_lifeexpectancy.xlsx
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="H2">
-        <v>0.625</v>
+        <v>0.7352941176470651</v>
       </c>
       <c r="I2">
         <v>2023</v>
@@ -482,7 +482,7 @@
         <v>2015</v>
       </c>
       <c r="O2">
-        <v>77</v>
+        <v>76.76000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="H3">
-        <v>1.385416666666654</v>
+        <v>1.405859708060271</v>
       </c>
       <c r="I3">
         <v>2023</v>
@@ -536,7 +536,7 @@
         <v>2015</v>
       </c>
       <c r="O3">
-        <v>65.07500000000002</v>
+        <v>65.03438746424041</v>
       </c>
     </row>
     <row r="4">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="H4">
-        <v>1.208333333333329</v>
+        <v>1.243398001283063</v>
       </c>
       <c r="I4">
         <v>2023</v>
@@ -590,7 +590,7 @@
         <v>2015</v>
       </c>
       <c r="O4">
-        <v>64.10000000000001</v>
+        <v>63.96257864863126</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="H5">
-        <v>0.75</v>
+        <v>0.8823529411764781</v>
       </c>
       <c r="I5">
         <v>2023</v>
@@ -644,7 +644,7 @@
         <v>2015</v>
       </c>
       <c r="O5">
-        <v>80</v>
+        <v>79.76000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -672,17 +672,11 @@
           <t>AND</t>
         </is>
       </c>
-      <c r="H6">
-        <v>-0.625</v>
-      </c>
       <c r="I6">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J6">
-        <v>84</v>
-      </c>
-      <c r="K6">
-        <v>84.5</v>
+        <v>84.188</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -693,12 +687,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N6">
-        <v>2015</v>
-      </c>
-      <c r="O6">
-        <v>85.30000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +715,7 @@
         </is>
       </c>
       <c r="H7">
-        <v>0.6875</v>
+        <v>3.397321428571427</v>
       </c>
       <c r="I7">
         <v>2023</v>
@@ -752,7 +740,7 @@
         <v>2015</v>
       </c>
       <c r="O7">
-        <v>83.15000000000001</v>
+        <v>82.56619047619049</v>
       </c>
     </row>
     <row r="8">
@@ -781,7 +769,7 @@
         </is>
       </c>
       <c r="H8">
-        <v>0.5</v>
+        <v>0.5882352941176521</v>
       </c>
       <c r="I8">
         <v>2023</v>
@@ -806,7 +794,7 @@
         <v>2015</v>
       </c>
       <c r="O8">
-        <v>78.2</v>
+        <v>77.95999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -835,7 +823,7 @@
         </is>
       </c>
       <c r="H9">
-        <v>0.9375</v>
+        <v>1.102941176470598</v>
       </c>
       <c r="I9">
         <v>2023</v>
@@ -860,7 +848,7 @@
         <v>2015</v>
       </c>
       <c r="O9">
-        <v>75.8</v>
+        <v>75.56</v>
       </c>
     </row>
     <row r="10">
@@ -889,7 +877,7 @@
         </is>
       </c>
       <c r="H10">
-        <v>0.125</v>
+        <v>0.147058823529413</v>
       </c>
       <c r="I10">
         <v>2023</v>
@@ -914,7 +902,7 @@
         <v>2015</v>
       </c>
       <c r="O10">
-        <v>74.3</v>
+        <v>74.06</v>
       </c>
     </row>
     <row r="11">
@@ -943,7 +931,7 @@
         </is>
       </c>
       <c r="H11">
-        <v>0.4375</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I11">
         <v>2023</v>
@@ -968,7 +956,7 @@
         <v>2015</v>
       </c>
       <c r="O11">
-        <v>78.5</v>
+        <v>78.26000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -996,17 +984,11 @@
           <t>AUS</t>
         </is>
       </c>
-      <c r="H12">
-        <v>1.625</v>
-      </c>
       <c r="I12">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J12">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="K12">
-        <v>82.60000000000001</v>
+        <v>84.07299999999999</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1017,12 +999,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N12">
-        <v>2015</v>
-      </c>
-      <c r="O12">
-        <v>83.40000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -1051,7 +1027,7 @@
         </is>
       </c>
       <c r="H13">
-        <v>0.5</v>
+        <v>0.8273185148185185</v>
       </c>
       <c r="I13">
         <v>2023</v>
@@ -1076,7 +1052,7 @@
         <v>2015</v>
       </c>
       <c r="O13">
-        <v>82.7</v>
+        <v>82.12162726162727</v>
       </c>
     </row>
     <row r="14">
@@ -1105,7 +1081,7 @@
         </is>
       </c>
       <c r="H14">
-        <v>1.312500000000002</v>
+        <v>1.531862745098051</v>
       </c>
       <c r="I14">
         <v>2023</v>
@@ -1130,7 +1106,7 @@
         <v>2015</v>
       </c>
       <c r="O14">
-        <v>73.90000000000001</v>
+        <v>73.67666666666666</v>
       </c>
     </row>
     <row r="15">
@@ -1159,7 +1135,7 @@
         </is>
       </c>
       <c r="H15">
-        <v>1.125</v>
+        <v>1.174950375558723</v>
       </c>
       <c r="I15">
         <v>2023</v>
@@ -1184,7 +1160,7 @@
         <v>2015</v>
       </c>
       <c r="O15">
-        <v>63.3</v>
+        <v>63.21308012490614</v>
       </c>
     </row>
     <row r="16">
@@ -1213,7 +1189,7 @@
         </is>
       </c>
       <c r="H16">
-        <v>0.75</v>
+        <v>1.216207403707404</v>
       </c>
       <c r="I16">
         <v>2023</v>
@@ -1238,7 +1214,7 @@
         <v>2015</v>
       </c>
       <c r="O16">
-        <v>82.5</v>
+        <v>81.9381451881452</v>
       </c>
     </row>
     <row r="17">
@@ -1267,7 +1243,7 @@
         </is>
       </c>
       <c r="H17">
-        <v>0.53125</v>
+        <v>0.4992581392893456</v>
       </c>
       <c r="I17">
         <v>2023</v>
@@ -1292,7 +1268,7 @@
         <v>2015</v>
       </c>
       <c r="O17">
-        <v>62.3</v>
+        <v>62.37024723912776</v>
       </c>
     </row>
     <row r="18">
@@ -1321,7 +1297,7 @@
         </is>
       </c>
       <c r="H18">
-        <v>0.7125000000000004</v>
+        <v>0.6760797086414065</v>
       </c>
       <c r="I18">
         <v>2023</v>
@@ -1346,7 +1322,7 @@
         <v>2015</v>
       </c>
       <c r="O18">
-        <v>62.01999999999998</v>
+        <v>62.11497409598651</v>
       </c>
     </row>
     <row r="19">
@@ -1375,7 +1351,7 @@
         </is>
       </c>
       <c r="H19">
-        <v>2.625000000000002</v>
+        <v>2.966266769865857</v>
       </c>
       <c r="I19">
         <v>2023</v>
@@ -1400,7 +1376,7 @@
         <v>2015</v>
       </c>
       <c r="O19">
-        <v>72.10000000000001</v>
+        <v>71.99210526315788</v>
       </c>
     </row>
     <row r="20">
@@ -1429,7 +1405,7 @@
         </is>
       </c>
       <c r="H20">
-        <v>0.625</v>
+        <v>0.7352941176470651</v>
       </c>
       <c r="I20">
         <v>2023</v>
@@ -1454,7 +1430,7 @@
         <v>2015</v>
       </c>
       <c r="O20">
-        <v>76.2</v>
+        <v>75.95999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -1483,7 +1459,7 @@
         </is>
       </c>
       <c r="H21">
-        <v>0.625</v>
+        <v>0.7988445378151248</v>
       </c>
       <c r="I21">
         <v>2023</v>
@@ -1508,7 +1484,7 @@
         <v>2015</v>
       </c>
       <c r="O21">
-        <v>81.90000000000001</v>
+        <v>81.51634453781513</v>
       </c>
     </row>
     <row r="22">
@@ -1537,7 +1513,7 @@
         </is>
       </c>
       <c r="H22">
-        <v>0.5</v>
+        <v>0.5882352941176521</v>
       </c>
       <c r="I22">
         <v>2023</v>
@@ -1562,7 +1538,7 @@
         <v>2015</v>
       </c>
       <c r="O22">
-        <v>75.40000000000001</v>
+        <v>75.16</v>
       </c>
     </row>
     <row r="23">
@@ -1591,7 +1567,7 @@
         </is>
       </c>
       <c r="H23">
-        <v>0.4375</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I23">
         <v>2023</v>
@@ -1616,7 +1592,7 @@
         <v>2015</v>
       </c>
       <c r="O23">
-        <v>78.7</v>
+        <v>78.45999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -1645,7 +1621,7 @@
         </is>
       </c>
       <c r="H24">
-        <v>0.375</v>
+        <v>0.4411764705882391</v>
       </c>
       <c r="I24">
         <v>2023</v>
@@ -1670,7 +1646,7 @@
         <v>2015</v>
       </c>
       <c r="O24">
-        <v>75.40000000000001</v>
+        <v>75.16</v>
       </c>
     </row>
     <row r="25">
@@ -1699,7 +1675,7 @@
         </is>
       </c>
       <c r="H25">
-        <v>1.250000000000002</v>
+        <v>1.429738562091512</v>
       </c>
       <c r="I25">
         <v>2023</v>
@@ -1724,7 +1700,7 @@
         <v>2015</v>
       </c>
       <c r="O25">
-        <v>73.2</v>
+        <v>73.01555555555555</v>
       </c>
     </row>
     <row r="26">
@@ -1753,7 +1729,7 @@
         </is>
       </c>
       <c r="H26">
-        <v>1.25</v>
+        <v>2.010587655808244</v>
       </c>
       <c r="I26">
         <v>2023</v>
@@ -1778,7 +1754,7 @@
         <v>2015</v>
       </c>
       <c r="O26">
-        <v>81.90000000000001</v>
+        <v>81.51634453781513</v>
       </c>
     </row>
     <row r="27">
@@ -1807,7 +1783,7 @@
         </is>
       </c>
       <c r="H27">
-        <v>0.6666666666666607</v>
+        <v>0.7238015607580905</v>
       </c>
       <c r="I27">
         <v>2023</v>
@@ -1832,7 +1808,7 @@
         <v>2015</v>
       </c>
       <c r="O27">
-        <v>69.13333333333335</v>
+        <v>69.09045707915271</v>
       </c>
     </row>
     <row r="28">
@@ -1861,7 +1837,7 @@
         </is>
       </c>
       <c r="H28">
-        <v>0.4375</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I28">
         <v>2023</v>
@@ -1886,7 +1862,7 @@
         <v>2015</v>
       </c>
       <c r="O28">
-        <v>76.7</v>
+        <v>76.45999999999999</v>
       </c>
     </row>
     <row r="29">
@@ -1915,7 +1891,7 @@
         </is>
       </c>
       <c r="H29">
-        <v>0.0625</v>
+        <v>0.07352941176470651</v>
       </c>
       <c r="I29">
         <v>2023</v>
@@ -1940,7 +1916,7 @@
         <v>2015</v>
       </c>
       <c r="O29">
-        <v>77.7</v>
+        <v>77.45999999999999</v>
       </c>
     </row>
     <row r="30">
@@ -1969,7 +1945,7 @@
         </is>
       </c>
       <c r="H30">
-        <v>0.25</v>
+        <v>0.294117647058826</v>
       </c>
       <c r="I30">
         <v>2023</v>
@@ -1994,7 +1970,7 @@
         <v>2015</v>
       </c>
       <c r="O30">
-        <v>76.5</v>
+        <v>76.25999999999999</v>
       </c>
     </row>
     <row r="31">
@@ -2023,7 +1999,7 @@
         </is>
       </c>
       <c r="H31">
-        <v>1.375</v>
+        <v>1.522187822497425</v>
       </c>
       <c r="I31">
         <v>2023</v>
@@ -2048,7 +2024,7 @@
         <v>2015</v>
       </c>
       <c r="O31">
-        <v>72.40000000000001</v>
+        <v>72.27157894736841</v>
       </c>
     </row>
     <row r="32">
@@ -2077,7 +2053,7 @@
         </is>
       </c>
       <c r="H32">
-        <v>2.645833333333307</v>
+        <v>2.7145758754721</v>
       </c>
       <c r="I32">
         <v>2023</v>
@@ -2102,7 +2078,7 @@
         <v>2015</v>
       </c>
       <c r="O32">
-        <v>65.75000000000003</v>
+        <v>65.77251959141429</v>
       </c>
     </row>
     <row r="33">
@@ -2131,7 +2107,7 @@
         </is>
       </c>
       <c r="H33">
-        <v>1.37500000000002</v>
+        <v>1.390676909061492</v>
       </c>
       <c r="I33">
         <v>2023</v>
@@ -2156,7 +2132,7 @@
         <v>2015</v>
       </c>
       <c r="O33">
-        <v>55.90000000000001</v>
+        <v>55.9107450980392</v>
       </c>
     </row>
     <row r="34">
@@ -2185,7 +2161,7 @@
         </is>
       </c>
       <c r="H34">
-        <v>0.4375</v>
+        <v>1.369543650793648</v>
       </c>
       <c r="I34">
         <v>2023</v>
@@ -2210,7 +2186,7 @@
         <v>2015</v>
       </c>
       <c r="O34">
-        <v>83.05000000000001</v>
+        <v>82.47718253968254</v>
       </c>
     </row>
     <row r="35">
@@ -2238,17 +2214,11 @@
           <t>CHE</t>
         </is>
       </c>
-      <c r="H35">
-        <v>1.5</v>
-      </c>
       <c r="I35">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J35">
-        <v>84</v>
-      </c>
-      <c r="K35">
-        <v>82.80000000000001</v>
+        <v>84.08799999999999</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -2259,12 +2229,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N35">
-        <v>2015</v>
-      </c>
-      <c r="O35">
-        <v>83.60000000000001</v>
       </c>
     </row>
     <row r="36">
@@ -2293,7 +2257,7 @@
         </is>
       </c>
       <c r="H36">
-        <v>-0.0625</v>
+        <v>-0.0961538461538467</v>
       </c>
       <c r="I36">
         <v>2023</v>
@@ -2318,7 +2282,7 @@
         <v>2015</v>
       </c>
       <c r="O36">
-        <v>82.90000000000001</v>
+        <v>82.33352813852815</v>
       </c>
     </row>
     <row r="37">
@@ -2347,7 +2311,7 @@
         </is>
       </c>
       <c r="H37">
-        <v>0.75</v>
+        <v>0.930147058823529</v>
       </c>
       <c r="I37">
         <v>2023</v>
@@ -2372,7 +2336,7 @@
         <v>2015</v>
       </c>
       <c r="O37">
-        <v>81.60000000000001</v>
+        <v>81.27823529411764</v>
       </c>
     </row>
     <row r="38">
@@ -2401,7 +2365,7 @@
         </is>
       </c>
       <c r="H38">
-        <v>0.625</v>
+        <v>0.7352941176470651</v>
       </c>
       <c r="I38">
         <v>2023</v>
@@ -2426,7 +2390,7 @@
         <v>2015</v>
       </c>
       <c r="O38">
-        <v>78.60000000000001</v>
+        <v>78.36</v>
       </c>
     </row>
     <row r="39">
@@ -2455,7 +2419,7 @@
         </is>
       </c>
       <c r="H39">
-        <v>1.087500000000002</v>
+        <v>1.068173725735431</v>
       </c>
       <c r="I39">
         <v>2023</v>
@@ -2480,7 +2444,7 @@
         <v>2015</v>
       </c>
       <c r="O39">
-        <v>61.61999999999998</v>
+        <v>61.6872979757055</v>
       </c>
     </row>
     <row r="40">
@@ -2509,7 +2473,7 @@
         </is>
       </c>
       <c r="H40">
-        <v>1.25</v>
+        <v>1.291921582646211</v>
       </c>
       <c r="I40">
         <v>2023</v>
@@ -2534,7 +2498,7 @@
         <v>2015</v>
       </c>
       <c r="O40">
-        <v>62.90000000000001</v>
+        <v>62.87657676634868</v>
       </c>
     </row>
     <row r="41">
@@ -2563,7 +2527,7 @@
         </is>
       </c>
       <c r="H41">
-        <v>0.9875000000000007</v>
+        <v>0.9570626146243164</v>
       </c>
       <c r="I41">
         <v>2023</v>
@@ -2588,7 +2552,7 @@
         <v>2015</v>
       </c>
       <c r="O41">
-        <v>61.93999999999997</v>
+        <v>62.0305296515421</v>
       </c>
     </row>
     <row r="42">
@@ -2617,7 +2581,7 @@
         </is>
       </c>
       <c r="H42">
-        <v>0.8645833333333215</v>
+        <v>0.8322231549612429</v>
       </c>
       <c r="I42">
         <v>2023</v>
@@ -2642,7 +2606,7 @@
         <v>2015</v>
       </c>
       <c r="O42">
-        <v>66.12500000000004</v>
+        <v>66.18271668461097</v>
       </c>
     </row>
     <row r="43">
@@ -2671,7 +2635,7 @@
         </is>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>1.176470588235304</v>
       </c>
       <c r="I43">
         <v>2023</v>
@@ -2696,7 +2660,7 @@
         <v>2015</v>
       </c>
       <c r="O43">
-        <v>77.7</v>
+        <v>77.45999999999999</v>
       </c>
     </row>
     <row r="44">
@@ -2725,7 +2689,7 @@
         </is>
       </c>
       <c r="H44">
-        <v>0.9583333333333197</v>
+        <v>0.9813148961073708</v>
       </c>
       <c r="I44">
         <v>2023</v>
@@ -2750,7 +2714,7 @@
         <v>2015</v>
       </c>
       <c r="O44">
-        <v>66.90000000000001</v>
+        <v>66.84035982440808</v>
       </c>
     </row>
     <row r="45">
@@ -2779,7 +2743,7 @@
         </is>
       </c>
       <c r="H45">
-        <v>1.25</v>
+        <v>1.47058823529413</v>
       </c>
       <c r="I45">
         <v>2023</v>
@@ -2804,7 +2768,7 @@
         <v>2015</v>
       </c>
       <c r="O45">
-        <v>75.7</v>
+        <v>75.45999999999999</v>
       </c>
     </row>
     <row r="46">
@@ -2833,7 +2797,7 @@
         </is>
       </c>
       <c r="H46">
-        <v>0.25</v>
+        <v>0.3079044117647065</v>
       </c>
       <c r="I46">
         <v>2023</v>
@@ -2858,7 +2822,7 @@
         <v>2015</v>
       </c>
       <c r="O46">
-        <v>82</v>
+        <v>81.59281512605044</v>
       </c>
     </row>
     <row r="47">
@@ -2887,7 +2851,7 @@
         </is>
       </c>
       <c r="H47">
-        <v>0.25</v>
+        <v>0.294117647058826</v>
       </c>
       <c r="I47">
         <v>2023</v>
@@ -2912,7 +2876,7 @@
         <v>2015</v>
       </c>
       <c r="O47">
-        <v>79.30000000000001</v>
+        <v>79.06</v>
       </c>
     </row>
     <row r="48">
@@ -2941,7 +2905,7 @@
         </is>
       </c>
       <c r="H48">
-        <v>0.1875</v>
+        <v>0.2205882352941195</v>
       </c>
       <c r="I48">
         <v>2023</v>
@@ -2966,7 +2930,7 @@
         <v>2015</v>
       </c>
       <c r="O48">
-        <v>78.10000000000001</v>
+        <v>77.86</v>
       </c>
     </row>
     <row r="49">
@@ -2995,7 +2959,7 @@
         </is>
       </c>
       <c r="H49">
-        <v>1.4375</v>
+        <v>1.69117647058825</v>
       </c>
       <c r="I49">
         <v>2023</v>
@@ -3020,7 +2984,7 @@
         <v>2015</v>
       </c>
       <c r="O49">
-        <v>79.7</v>
+        <v>79.45999999999999</v>
       </c>
     </row>
     <row r="50">
@@ -3049,7 +3013,7 @@
         </is>
       </c>
       <c r="H50">
-        <v>0.0625</v>
+        <v>0.0961538461538467</v>
       </c>
       <c r="I50">
         <v>2023</v>
@@ -3074,7 +3038,7 @@
         <v>2015</v>
       </c>
       <c r="O50">
-        <v>82.85000000000001</v>
+        <v>82.28527000777002</v>
       </c>
     </row>
     <row r="51">
@@ -3103,7 +3067,7 @@
         </is>
       </c>
       <c r="H51">
-        <v>0.75</v>
+        <v>0.8823529411764781</v>
       </c>
       <c r="I51">
         <v>2023</v>
@@ -3128,7 +3092,7 @@
         <v>2015</v>
       </c>
       <c r="O51">
-        <v>80.2</v>
+        <v>79.95999999999999</v>
       </c>
     </row>
     <row r="52">
@@ -3157,7 +3121,7 @@
         </is>
       </c>
       <c r="H52">
-        <v>0.5</v>
+        <v>0.662946428571427</v>
       </c>
       <c r="I52">
         <v>2023</v>
@@ -3182,7 +3146,7 @@
         <v>2015</v>
       </c>
       <c r="O52">
-        <v>82.2</v>
+        <v>81.73570970695971</v>
       </c>
     </row>
     <row r="53">
@@ -3211,7 +3175,7 @@
         </is>
       </c>
       <c r="H53">
-        <v>1.229166666666654</v>
+        <v>1.23694078914135</v>
       </c>
       <c r="I53">
         <v>2023</v>
@@ -3236,7 +3200,7 @@
         <v>2015</v>
       </c>
       <c r="O53">
-        <v>65.45000000000003</v>
+        <v>65.44513520950902</v>
       </c>
     </row>
     <row r="54">
@@ -3265,7 +3229,7 @@
         </is>
       </c>
       <c r="H54">
-        <v>0.6875</v>
+        <v>0.7039473684210531</v>
       </c>
       <c r="I54">
         <v>2023</v>
@@ -3290,7 +3254,7 @@
         <v>2015</v>
       </c>
       <c r="O54">
-        <v>71.60000000000001</v>
+        <v>71.54210526315789</v>
       </c>
     </row>
     <row r="55">
@@ -3319,7 +3283,7 @@
         </is>
       </c>
       <c r="H55">
-        <v>0.75</v>
+        <v>1.108568514818515</v>
       </c>
       <c r="I55">
         <v>2023</v>
@@ -3344,7 +3308,7 @@
         <v>2015</v>
       </c>
       <c r="O55">
-        <v>82.30000000000001</v>
+        <v>81.80445970695972</v>
       </c>
     </row>
     <row r="56">
@@ -3373,7 +3337,7 @@
         </is>
       </c>
       <c r="H56">
-        <v>0.4375000000000018</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I56">
         <v>2023</v>
@@ -3398,7 +3362,7 @@
         <v>2015</v>
       </c>
       <c r="O56">
-        <v>74.60000000000001</v>
+        <v>74.36</v>
       </c>
     </row>
     <row r="57">
@@ -3427,7 +3391,7 @@
         </is>
       </c>
       <c r="H57">
-        <v>0.6875</v>
+        <v>0.8088235294117716</v>
       </c>
       <c r="I57">
         <v>2023</v>
@@ -3452,7 +3416,7 @@
         <v>2015</v>
       </c>
       <c r="O57">
-        <v>76.80000000000001</v>
+        <v>76.56</v>
       </c>
     </row>
     <row r="58">
@@ -3481,7 +3445,7 @@
         </is>
       </c>
       <c r="H58">
-        <v>0.75</v>
+        <v>0.8823529411764781</v>
       </c>
       <c r="I58">
         <v>2023</v>
@@ -3506,7 +3470,7 @@
         <v>2015</v>
       </c>
       <c r="O58">
-        <v>77.80000000000001</v>
+        <v>77.56</v>
       </c>
     </row>
     <row r="59">
@@ -3535,7 +3499,7 @@
         </is>
       </c>
       <c r="H59">
-        <v>0.9375</v>
+        <v>0.9777046783625742</v>
       </c>
       <c r="I59">
         <v>2023</v>
@@ -3560,7 +3524,7 @@
         <v>2015</v>
       </c>
       <c r="O59">
-        <v>71.7</v>
+        <v>71.6321052631579</v>
       </c>
     </row>
     <row r="60">
@@ -3589,7 +3553,7 @@
         </is>
       </c>
       <c r="H60">
-        <v>1.20833333333332</v>
+        <v>1.321188688317632</v>
       </c>
       <c r="I60">
         <v>2023</v>
@@ -3614,7 +3578,7 @@
         <v>2015</v>
       </c>
       <c r="O60">
-        <v>68.26666666666669</v>
+        <v>68.00070902277795</v>
       </c>
     </row>
     <row r="61">
@@ -3642,17 +3606,11 @@
           <t>ESP</t>
         </is>
       </c>
-      <c r="H61">
-        <v>1.375</v>
-      </c>
       <c r="I61">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J61">
-        <v>83.7</v>
-      </c>
-      <c r="K61">
-        <v>82.60000000000001</v>
+        <v>83.79900000000001</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -3663,12 +3621,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N61">
-        <v>2015</v>
-      </c>
-      <c r="O61">
-        <v>83.40000000000001</v>
       </c>
     </row>
     <row r="62">
@@ -3697,7 +3649,7 @@
         </is>
       </c>
       <c r="H62">
-        <v>0.9375</v>
+        <v>1.102941176470598</v>
       </c>
       <c r="I62">
         <v>2023</v>
@@ -3722,7 +3674,7 @@
         <v>2015</v>
       </c>
       <c r="O62">
-        <v>79.30000000000001</v>
+        <v>79.06</v>
       </c>
     </row>
     <row r="63">
@@ -3751,7 +3703,7 @@
         </is>
       </c>
       <c r="H63">
-        <v>1.520833333333313</v>
+        <v>1.557555359755922</v>
       </c>
       <c r="I63">
         <v>2023</v>
@@ -3776,7 +3728,7 @@
         <v>2015</v>
       </c>
       <c r="O63">
-        <v>66.05000000000004</v>
+        <v>66.10036374343451</v>
       </c>
     </row>
     <row r="64">
@@ -3805,7 +3757,7 @@
         </is>
       </c>
       <c r="H64">
-        <v>0.3125</v>
+        <v>0.5237470862470879</v>
       </c>
       <c r="I64">
         <v>2023</v>
@@ -3830,7 +3782,7 @@
         <v>2015</v>
       </c>
       <c r="O64">
-        <v>82.80000000000001</v>
+        <v>82.23142385392386</v>
       </c>
     </row>
     <row r="65">
@@ -3859,7 +3811,7 @@
         </is>
       </c>
       <c r="H65">
-        <v>0.3333333333333286</v>
+        <v>0.3774928774928767</v>
       </c>
       <c r="I65">
         <v>2023</v>
@@ -3884,7 +3836,7 @@
         <v>2015</v>
       </c>
       <c r="O65">
-        <v>68.6666666666667</v>
+        <v>68.50207977207975</v>
       </c>
     </row>
     <row r="66">
@@ -3912,17 +3864,11 @@
           <t>FRA</t>
         </is>
       </c>
-      <c r="H66">
-        <v>1.1875</v>
-      </c>
       <c r="I66">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J66">
-        <v>83.30000000000001</v>
-      </c>
-      <c r="K66">
-        <v>82.10000000000001</v>
+        <v>83.458</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -3933,12 +3879,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N66">
-        <v>2015</v>
-      </c>
-      <c r="O66">
-        <v>83.15000000000001</v>
       </c>
     </row>
     <row r="67">
@@ -3967,7 +3907,7 @@
         </is>
       </c>
       <c r="H67">
-        <v>0.5</v>
+        <v>0.5882352941176521</v>
       </c>
       <c r="I67">
         <v>2023</v>
@@ -3992,7 +3932,7 @@
         <v>2015</v>
       </c>
       <c r="O67">
-        <v>81</v>
+        <v>80.74470588235295</v>
       </c>
     </row>
     <row r="68">
@@ -4021,7 +3961,7 @@
         </is>
       </c>
       <c r="H68">
-        <v>0.7916666666666554</v>
+        <v>0.8516974723871229</v>
       </c>
       <c r="I68">
         <v>2023</v>
@@ -4046,7 +3986,7 @@
         <v>2015</v>
       </c>
       <c r="O68">
-        <v>67.7</v>
+        <v>67.50045120907191</v>
       </c>
     </row>
     <row r="69">
@@ -4075,7 +4015,7 @@
         </is>
       </c>
       <c r="H69">
-        <v>0.8541666666666554</v>
+        <v>0.9811131903523265</v>
       </c>
       <c r="I69">
         <v>2023</v>
@@ -4100,7 +4040,7 @@
         <v>2015</v>
       </c>
       <c r="O69">
-        <v>68.53333333333335</v>
+        <v>68.33475172975173</v>
       </c>
     </row>
     <row r="70">
@@ -4129,7 +4069,7 @@
         </is>
       </c>
       <c r="H70">
-        <v>0.25</v>
+        <v>0.3392857142857117</v>
       </c>
       <c r="I70">
         <v>2023</v>
@@ -4154,7 +4094,7 @@
         <v>2015</v>
       </c>
       <c r="O70">
-        <v>82.5</v>
+        <v>81.9381451881452</v>
       </c>
     </row>
     <row r="71">
@@ -4183,7 +4123,7 @@
         </is>
       </c>
       <c r="H71">
-        <v>0.8125000000000018</v>
+        <v>0.9558823529411846</v>
       </c>
       <c r="I71">
         <v>2023</v>
@@ -4208,7 +4148,7 @@
         <v>2015</v>
       </c>
       <c r="O71">
-        <v>74.8</v>
+        <v>74.56</v>
       </c>
     </row>
     <row r="72">
@@ -4237,7 +4177,7 @@
         </is>
       </c>
       <c r="H72">
-        <v>0.8958333333333233</v>
+        <v>0.8839714404823535</v>
       </c>
       <c r="I72">
         <v>2023</v>
@@ -4262,7 +4202,7 @@
         <v>2015</v>
       </c>
       <c r="O72">
-        <v>65.75000000000003</v>
+        <v>65.77251959141429</v>
       </c>
     </row>
     <row r="73">
@@ -4290,17 +4230,11 @@
           <t>GIB</t>
         </is>
       </c>
-      <c r="H73">
-        <v>1.125</v>
-      </c>
       <c r="I73">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J73">
-        <v>83.60000000000001</v>
-      </c>
-      <c r="K73">
-        <v>82.7</v>
+        <v>83.63</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -4311,12 +4245,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N73">
-        <v>2015</v>
-      </c>
-      <c r="O73">
-        <v>83.5</v>
       </c>
     </row>
     <row r="74">
@@ -4345,7 +4273,7 @@
         </is>
       </c>
       <c r="H74">
-        <v>0.8125000000000036</v>
+        <v>0.8009508350700649</v>
       </c>
       <c r="I74">
         <v>2023</v>
@@ -4370,7 +4298,7 @@
         <v>2015</v>
       </c>
       <c r="O74">
-        <v>61.3</v>
+        <v>61.34427440094651</v>
       </c>
     </row>
     <row r="75">
@@ -4399,7 +4327,7 @@
         </is>
       </c>
       <c r="H75">
-        <v>1.124999999999988</v>
+        <v>1.124392896421046</v>
       </c>
       <c r="I75">
         <v>2023</v>
@@ -4424,7 +4352,7 @@
         <v>2015</v>
       </c>
       <c r="O75">
-        <v>65.60000000000001</v>
+        <v>65.61140848030317</v>
       </c>
     </row>
     <row r="76">
@@ -4453,7 +4381,7 @@
         </is>
       </c>
       <c r="H76">
-        <v>1.281249999999998</v>
+        <v>1.32312328108457</v>
       </c>
       <c r="I76">
         <v>2023</v>
@@ -4478,7 +4406,7 @@
         <v>2015</v>
       </c>
       <c r="O76">
-        <v>63.3</v>
+        <v>63.21308012490614</v>
       </c>
     </row>
     <row r="77">
@@ -4507,7 +4435,7 @@
         </is>
       </c>
       <c r="H77">
-        <v>0.96875</v>
+        <v>1.025414951633053</v>
       </c>
       <c r="I77">
         <v>2023</v>
@@ -4532,7 +4460,7 @@
         <v>2015</v>
       </c>
       <c r="O77">
-        <v>63.8</v>
+        <v>63.63087133155809</v>
       </c>
     </row>
     <row r="78">
@@ -4561,7 +4489,7 @@
         </is>
       </c>
       <c r="H78">
-        <v>0.6875</v>
+        <v>1.030443514818515</v>
       </c>
       <c r="I78">
         <v>2023</v>
@@ -4586,7 +4514,7 @@
         <v>2015</v>
       </c>
       <c r="O78">
-        <v>82.40000000000001</v>
+        <v>81.87320970695973</v>
       </c>
     </row>
     <row r="79">
@@ -4615,7 +4543,7 @@
         </is>
       </c>
       <c r="H79">
-        <v>0.125</v>
+        <v>0.147058823529413</v>
       </c>
       <c r="I79">
         <v>2023</v>
@@ -4640,7 +4568,7 @@
         <v>2015</v>
       </c>
       <c r="O79">
-        <v>76.60000000000001</v>
+        <v>76.36</v>
       </c>
     </row>
     <row r="80">
@@ -4694,7 +4622,7 @@
         <v>2015</v>
       </c>
       <c r="O80">
-        <v>71.8</v>
+        <v>71.7221052631579</v>
       </c>
     </row>
     <row r="81">
@@ -4723,7 +4651,7 @@
         </is>
       </c>
       <c r="H81">
-        <v>1.0625</v>
+        <v>1.162280701754389</v>
       </c>
       <c r="I81">
         <v>2023</v>
@@ -4748,7 +4676,7 @@
         <v>2015</v>
       </c>
       <c r="O81">
-        <v>72.5</v>
+        <v>72.36631578947369</v>
       </c>
     </row>
     <row r="82">
@@ -4777,7 +4705,7 @@
         </is>
       </c>
       <c r="H82">
-        <v>0.5</v>
+        <v>0.5882352941176521</v>
       </c>
       <c r="I82">
         <v>2023</v>
@@ -4802,7 +4730,7 @@
         <v>2015</v>
       </c>
       <c r="O82">
-        <v>78</v>
+        <v>77.76000000000001</v>
       </c>
     </row>
     <row r="83">
@@ -4831,7 +4759,7 @@
         </is>
       </c>
       <c r="H83">
-        <v>1.45833333333333</v>
+        <v>1.415624411820072</v>
       </c>
       <c r="I83">
         <v>2023</v>
@@ -4856,7 +4784,7 @@
         <v>2015</v>
       </c>
       <c r="O83">
-        <v>69.46666666666665</v>
+        <v>69.51675098814229</v>
       </c>
     </row>
     <row r="84">
@@ -4884,17 +4812,11 @@
           <t>HKG</t>
         </is>
       </c>
-      <c r="H84">
-        <v>1.75</v>
-      </c>
       <c r="I84">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J84">
-        <v>85.5</v>
-      </c>
-      <c r="K84">
-        <v>84.10000000000001</v>
+        <v>85.634</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -4905,12 +4827,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N84">
-        <v>2015</v>
-      </c>
-      <c r="O84">
-        <v>84.90000000000001</v>
       </c>
     </row>
     <row r="85">
@@ -4939,7 +4855,7 @@
         </is>
       </c>
       <c r="H85">
-        <v>1</v>
+        <v>1.119711042311666</v>
       </c>
       <c r="I85">
         <v>2023</v>
@@ -4964,7 +4880,7 @@
         <v>2015</v>
       </c>
       <c r="O85">
-        <v>72.90000000000001</v>
+        <v>72.73719298245614</v>
       </c>
     </row>
     <row r="86">
@@ -4993,7 +4909,7 @@
         </is>
       </c>
       <c r="H86">
-        <v>0.625</v>
+        <v>0.7352941176470651</v>
       </c>
       <c r="I86">
         <v>2023</v>
@@ -5018,7 +4934,7 @@
         <v>2015</v>
       </c>
       <c r="O86">
-        <v>79.2</v>
+        <v>78.95999999999999</v>
       </c>
     </row>
     <row r="87">
@@ -5047,7 +4963,7 @@
         </is>
       </c>
       <c r="H87">
-        <v>0.6458333333333268</v>
+        <v>0.6380036985468696</v>
       </c>
       <c r="I87">
         <v>2023</v>
@@ -5072,7 +4988,7 @@
         <v>2015</v>
       </c>
       <c r="O87">
-        <v>65.75000000000003</v>
+        <v>65.77251959141429</v>
       </c>
     </row>
     <row r="88">
@@ -5101,7 +5017,7 @@
         </is>
       </c>
       <c r="H88">
-        <v>0.8125</v>
+        <v>0.9558823529411846</v>
       </c>
       <c r="I88">
         <v>2023</v>
@@ -5126,7 +5042,7 @@
         <v>2015</v>
       </c>
       <c r="O88">
-        <v>77.30000000000001</v>
+        <v>77.06</v>
       </c>
     </row>
     <row r="89">
@@ -5155,7 +5071,7 @@
         </is>
       </c>
       <c r="H89">
-        <v>1</v>
+        <v>1.004542606516294</v>
       </c>
       <c r="I89">
         <v>2023</v>
@@ -5180,7 +5096,7 @@
         <v>2015</v>
       </c>
       <c r="O89">
-        <v>71.10000000000001</v>
+        <v>71.09309523809526</v>
       </c>
     </row>
     <row r="90">
@@ -5209,7 +5125,7 @@
         </is>
       </c>
       <c r="H90">
-        <v>0.4375</v>
+        <v>0.5428921568627452</v>
       </c>
       <c r="I90">
         <v>2023</v>
@@ -5234,7 +5150,7 @@
         <v>2015</v>
       </c>
       <c r="O90">
-        <v>81.90000000000001</v>
+        <v>81.51634453781513</v>
       </c>
     </row>
     <row r="91">
@@ -5263,7 +5179,7 @@
         </is>
       </c>
       <c r="H91">
-        <v>1.6875</v>
+        <v>1.737625313283214</v>
       </c>
       <c r="I91">
         <v>2023</v>
@@ -5288,7 +5204,7 @@
         <v>2015</v>
       </c>
       <c r="O91">
-        <v>70.90000000000001</v>
+        <v>70.91214285714285</v>
       </c>
     </row>
     <row r="92">
@@ -5317,7 +5233,7 @@
         </is>
       </c>
       <c r="H92">
-        <v>0.5625</v>
+        <v>1.23463689088689</v>
       </c>
       <c r="I92">
         <v>2023</v>
@@ -5342,7 +5258,7 @@
         <v>2015</v>
       </c>
       <c r="O92">
-        <v>82.85000000000001</v>
+        <v>82.28527000777002</v>
       </c>
     </row>
     <row r="93">
@@ -5371,7 +5287,7 @@
         </is>
       </c>
       <c r="H93">
-        <v>1.125</v>
+        <v>1.323529411764717</v>
       </c>
       <c r="I93">
         <v>2023</v>
@@ -5396,7 +5312,7 @@
         <v>2015</v>
       </c>
       <c r="O93">
-        <v>77.5</v>
+        <v>77.26000000000001</v>
       </c>
     </row>
     <row r="94">
@@ -5425,7 +5341,7 @@
         </is>
       </c>
       <c r="H94">
-        <v>1.4375</v>
+        <v>1.526315789473687</v>
       </c>
       <c r="I94">
         <v>2023</v>
@@ -5450,7 +5366,7 @@
         <v>2015</v>
       </c>
       <c r="O94">
-        <v>71.60000000000001</v>
+        <v>71.54210526315789</v>
       </c>
     </row>
     <row r="95">
@@ -5479,7 +5395,7 @@
         </is>
       </c>
       <c r="H95">
-        <v>0.375</v>
+        <v>1.366071428571427</v>
       </c>
       <c r="I95">
         <v>2023</v>
@@ -5504,7 +5420,7 @@
         <v>2015</v>
       </c>
       <c r="O95">
-        <v>83.2</v>
+        <v>82.61214285714287</v>
       </c>
     </row>
     <row r="96">
@@ -5533,7 +5449,7 @@
         </is>
       </c>
       <c r="H96">
-        <v>0.0625</v>
+        <v>0.2083333333333321</v>
       </c>
       <c r="I96">
         <v>2023</v>
@@ -5558,7 +5474,7 @@
         <v>2015</v>
       </c>
       <c r="O96">
-        <v>83.25</v>
+        <v>82.655</v>
       </c>
     </row>
     <row r="97">
@@ -5586,17 +5502,11 @@
           <t>ITA</t>
         </is>
       </c>
-      <c r="H97">
-        <v>1.4375</v>
-      </c>
       <c r="I97">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J97">
-        <v>83.7</v>
-      </c>
-      <c r="K97">
-        <v>82.5</v>
+        <v>83.869</v>
       </c>
       <c r="L97" t="inlineStr">
         <is>
@@ -5607,12 +5517,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N97">
-        <v>2015</v>
-      </c>
-      <c r="O97">
-        <v>83.35000000000001</v>
       </c>
     </row>
     <row r="98">
@@ -5641,7 +5545,7 @@
         </is>
       </c>
       <c r="H98">
-        <v>-0.4375</v>
+        <v>-0.4861111111111125</v>
       </c>
       <c r="I98">
         <v>2023</v>
@@ -5666,7 +5570,7 @@
         <v>2015</v>
       </c>
       <c r="O98">
-        <v>73.8</v>
+        <v>73.58222222222221</v>
       </c>
     </row>
     <row r="99">
@@ -5695,7 +5599,7 @@
         </is>
       </c>
       <c r="H99">
-        <v>1.6875</v>
+        <v>1.985294117647076</v>
       </c>
       <c r="I99">
         <v>2023</v>
@@ -5720,7 +5624,7 @@
         <v>2015</v>
       </c>
       <c r="O99">
-        <v>76.7</v>
+        <v>76.45999999999999</v>
       </c>
     </row>
     <row r="100">
@@ -5748,17 +5652,11 @@
           <t>JPN</t>
         </is>
       </c>
-      <c r="H100">
-        <v>1</v>
-      </c>
       <c r="I100">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J100">
-        <v>84.7</v>
-      </c>
-      <c r="K100">
-        <v>83.90000000000001</v>
+        <v>84.852</v>
       </c>
       <c r="L100" t="inlineStr">
         <is>
@@ -5769,12 +5667,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N100">
-        <v>2015</v>
-      </c>
-      <c r="O100">
-        <v>84.7</v>
       </c>
     </row>
     <row r="101">
@@ -5803,7 +5695,7 @@
         </is>
       </c>
       <c r="H101">
-        <v>1.500000000000002</v>
+        <v>1.740196078431385</v>
       </c>
       <c r="I101">
         <v>2023</v>
@@ -5828,7 +5720,7 @@
         <v>2015</v>
       </c>
       <c r="O101">
-        <v>73.60000000000001</v>
+        <v>73.39333333333335</v>
       </c>
     </row>
     <row r="102">
@@ -5857,7 +5749,7 @@
         </is>
       </c>
       <c r="H102">
-        <v>0.40625</v>
+        <v>0.4506649506649527</v>
       </c>
       <c r="I102">
         <v>2023</v>
@@ -5882,7 +5774,7 @@
         <v>2015</v>
       </c>
       <c r="O102">
-        <v>65.07500000000002</v>
+        <v>65.03438746424041</v>
       </c>
     </row>
     <row r="103">
@@ -5911,7 +5803,7 @@
         </is>
       </c>
       <c r="H103">
-        <v>1.5</v>
+        <v>1.52929197994988</v>
       </c>
       <c r="I103">
         <v>2023</v>
@@ -5936,7 +5828,7 @@
         <v>2015</v>
       </c>
       <c r="O103">
-        <v>70.90000000000001</v>
+        <v>70.91214285714285</v>
       </c>
     </row>
     <row r="104">
@@ -5965,7 +5857,7 @@
         </is>
       </c>
       <c r="H104">
-        <v>0.8125</v>
+        <v>0.8009085213032616</v>
       </c>
       <c r="I104">
         <v>2023</v>
@@ -5990,7 +5882,7 @@
         <v>2015</v>
       </c>
       <c r="O104">
-        <v>71</v>
+        <v>71.00261904761905</v>
       </c>
     </row>
     <row r="105">
@@ -6019,7 +5911,7 @@
         </is>
       </c>
       <c r="H105">
-        <v>0.2916666666666625</v>
+        <v>0.3110746214194489</v>
       </c>
       <c r="I105">
         <v>2023</v>
@@ -6044,7 +5936,7 @@
         <v>2015</v>
       </c>
       <c r="O105">
-        <v>68.2</v>
+        <v>67.91795040208835</v>
       </c>
     </row>
     <row r="106">
@@ -6073,7 +5965,7 @@
         </is>
       </c>
       <c r="H106">
-        <v>0.5625</v>
+        <v>0.6176900584795337</v>
       </c>
       <c r="I106">
         <v>2023</v>
@@ -6098,7 +5990,7 @@
         <v>2015</v>
       </c>
       <c r="O106">
-        <v>72.8</v>
+        <v>72.64771929824563</v>
       </c>
     </row>
     <row r="107">
@@ -6126,17 +6018,11 @@
           <t>KOR</t>
         </is>
       </c>
-      <c r="H107">
-        <v>2.1875</v>
-      </c>
       <c r="I107">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J107">
-        <v>84.30000000000001</v>
-      </c>
-      <c r="K107">
-        <v>82.5</v>
+        <v>84.434</v>
       </c>
       <c r="L107" t="inlineStr">
         <is>
@@ -6147,12 +6033,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N107">
-        <v>2015</v>
-      </c>
-      <c r="O107">
-        <v>83.35000000000001</v>
       </c>
     </row>
     <row r="108">
@@ -6181,7 +6061,7 @@
         </is>
       </c>
       <c r="H108">
-        <v>0.75</v>
+        <v>0.8823529411764781</v>
       </c>
       <c r="I108">
         <v>2023</v>
@@ -6206,7 +6086,7 @@
         <v>2015</v>
       </c>
       <c r="O108">
-        <v>80.80000000000001</v>
+        <v>80.55647058823529</v>
       </c>
     </row>
     <row r="109">
@@ -6235,7 +6115,7 @@
         </is>
       </c>
       <c r="H109">
-        <v>1.124999999999991</v>
+        <v>1.185427294122954</v>
       </c>
       <c r="I109">
         <v>2023</v>
@@ -6260,7 +6140,7 @@
         <v>2015</v>
       </c>
       <c r="O109">
-        <v>68.8</v>
+        <v>68.67245014245013</v>
       </c>
     </row>
     <row r="110">
@@ -6289,7 +6169,7 @@
         </is>
       </c>
       <c r="H110">
-        <v>-0.3125</v>
+        <v>-0.3676470588235325</v>
       </c>
       <c r="I110">
         <v>2023</v>
@@ -6314,7 +6194,7 @@
         <v>2015</v>
       </c>
       <c r="O110">
-        <v>79.90000000000001</v>
+        <v>79.66</v>
       </c>
     </row>
     <row r="111">
@@ -6343,7 +6223,7 @@
         </is>
       </c>
       <c r="H111">
-        <v>0.9375</v>
+        <v>0.9149639968677974</v>
       </c>
       <c r="I111">
         <v>2023</v>
@@ -6368,7 +6248,7 @@
         <v>2015</v>
       </c>
       <c r="O111">
-        <v>62.40000000000001</v>
+        <v>62.45433814821867</v>
       </c>
     </row>
     <row r="112">
@@ -6397,7 +6277,7 @@
         </is>
       </c>
       <c r="H112">
-        <v>-1.4375</v>
+        <v>-1.459847535505435</v>
       </c>
       <c r="I112">
         <v>2023</v>
@@ -6422,7 +6302,7 @@
         <v>2015</v>
       </c>
       <c r="O112">
-        <v>73.2</v>
+        <v>73.01555555555555</v>
       </c>
     </row>
     <row r="113">
@@ -6451,7 +6331,7 @@
         </is>
       </c>
       <c r="H113">
-        <v>-0.125</v>
+        <v>-0.147058823529413</v>
       </c>
       <c r="I113">
         <v>2023</v>
@@ -6476,7 +6356,7 @@
         <v>2015</v>
       </c>
       <c r="O113">
-        <v>74.5</v>
+        <v>74.25999999999999</v>
       </c>
     </row>
     <row r="114">
@@ -6504,17 +6384,11 @@
           <t>LIE</t>
         </is>
       </c>
-      <c r="H114">
-        <v>1</v>
-      </c>
       <c r="I114">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J114">
-        <v>83.60000000000001</v>
-      </c>
-      <c r="K114">
-        <v>82.80000000000001</v>
+        <v>83.748</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -6525,12 +6399,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N114">
-        <v>2015</v>
-      </c>
-      <c r="O114">
-        <v>83.60000000000001</v>
       </c>
     </row>
     <row r="115">
@@ -6559,7 +6427,7 @@
         </is>
       </c>
       <c r="H115">
-        <v>0.9375</v>
+        <v>1.102941176470598</v>
       </c>
       <c r="I115">
         <v>2023</v>
@@ -6584,7 +6452,7 @@
         <v>2015</v>
       </c>
       <c r="O115">
-        <v>77.60000000000001</v>
+        <v>77.36</v>
       </c>
     </row>
     <row r="116">
@@ -6613,7 +6481,7 @@
         </is>
       </c>
       <c r="H116">
-        <v>1.40000000000002</v>
+        <v>1.41518671298306</v>
       </c>
       <c r="I116">
         <v>2023</v>
@@ -6638,7 +6506,7 @@
         <v>2015</v>
       </c>
       <c r="O116">
-        <v>55.8</v>
+        <v>55.8146666666667</v>
       </c>
     </row>
     <row r="117">
@@ -6667,7 +6535,7 @@
         </is>
       </c>
       <c r="H117">
-        <v>0.9375</v>
+        <v>1.102941176470598</v>
       </c>
       <c r="I117">
         <v>2023</v>
@@ -6692,7 +6560,7 @@
         <v>2015</v>
       </c>
       <c r="O117">
-        <v>76.10000000000001</v>
+        <v>75.86</v>
       </c>
     </row>
     <row r="118">
@@ -6721,7 +6589,7 @@
         </is>
       </c>
       <c r="H118">
-        <v>0.5625</v>
+        <v>1.033171689421692</v>
       </c>
       <c r="I118">
         <v>2023</v>
@@ -6746,7 +6614,7 @@
         <v>2015</v>
       </c>
       <c r="O118">
-        <v>82.75</v>
+        <v>82.17877011877012</v>
       </c>
     </row>
     <row r="119">
@@ -6775,7 +6643,7 @@
         </is>
       </c>
       <c r="H119">
-        <v>0.9375</v>
+        <v>1.102941176470598</v>
       </c>
       <c r="I119">
         <v>2023</v>
@@ -6800,7 +6668,7 @@
         <v>2015</v>
       </c>
       <c r="O119">
-        <v>76.3</v>
+        <v>76.06</v>
       </c>
     </row>
     <row r="120">
@@ -6828,17 +6696,11 @@
           <t>MAC</t>
         </is>
       </c>
-      <c r="H120">
-        <v>0.25</v>
-      </c>
       <c r="I120">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J120">
-        <v>83.10000000000001</v>
-      </c>
-      <c r="K120">
-        <v>82.90000000000001</v>
+        <v>83.22799999999999</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
@@ -6849,12 +6711,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N120">
-        <v>2015</v>
-      </c>
-      <c r="O120">
-        <v>83.7</v>
       </c>
     </row>
     <row r="121">
@@ -6883,7 +6739,7 @@
         </is>
       </c>
       <c r="H121">
-        <v>0.25</v>
+        <v>0.294117647058826</v>
       </c>
       <c r="I121">
         <v>2023</v>
@@ -6908,7 +6764,7 @@
         <v>2015</v>
       </c>
       <c r="O121">
-        <v>81.40000000000001</v>
+        <v>81.10735294117647</v>
       </c>
     </row>
     <row r="122">
@@ -6937,7 +6793,7 @@
         </is>
       </c>
       <c r="H122">
-        <v>1.500000000000002</v>
+        <v>1.764705882352956</v>
       </c>
       <c r="I122">
         <v>2023</v>
@@ -6962,7 +6818,7 @@
         <v>2015</v>
       </c>
       <c r="O122">
-        <v>74.5</v>
+        <v>74.25999999999999</v>
       </c>
     </row>
     <row r="123">
@@ -6990,17 +6846,11 @@
           <t>MCO</t>
         </is>
       </c>
-      <c r="H123">
-        <v>0.5714285714285714</v>
-      </c>
       <c r="I123">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="J123">
-        <v>85.7</v>
-      </c>
-      <c r="K123">
-        <v>85.30000000000001</v>
+        <v>86.497</v>
       </c>
       <c r="L123" t="inlineStr">
         <is>
@@ -7011,12 +6861,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N123">
-        <v>2015</v>
-      </c>
-      <c r="O123">
-        <v>86</v>
       </c>
     </row>
     <row r="124">
@@ -7045,7 +6889,7 @@
         </is>
       </c>
       <c r="H124">
-        <v>0.6875</v>
+        <v>0.7072368421052637</v>
       </c>
       <c r="I124">
         <v>2023</v>
@@ -7070,7 +6914,7 @@
         <v>2015</v>
       </c>
       <c r="O124">
-        <v>71.7</v>
+        <v>71.6321052631579</v>
       </c>
     </row>
     <row r="125">
@@ -7099,7 +6943,7 @@
         </is>
       </c>
       <c r="H125">
-        <v>0.0625</v>
+        <v>0.07142857142857295</v>
       </c>
       <c r="I125">
         <v>2023</v>
@@ -7124,7 +6968,7 @@
         <v>2015</v>
       </c>
       <c r="O125">
-        <v>65.90000000000001</v>
+        <v>65.93823387712855</v>
       </c>
     </row>
     <row r="126">
@@ -7153,7 +6997,7 @@
         </is>
       </c>
       <c r="H126">
-        <v>1.5</v>
+        <v>1.792892156862756</v>
       </c>
       <c r="I126">
         <v>2023</v>
@@ -7178,7 +7022,7 @@
         <v>2015</v>
       </c>
       <c r="O126">
-        <v>80.2</v>
+        <v>79.95999999999999</v>
       </c>
     </row>
     <row r="127">
@@ -7207,7 +7051,7 @@
         </is>
       </c>
       <c r="H127">
-        <v>0.4375</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I127">
         <v>2023</v>
@@ -7232,7 +7076,7 @@
         <v>2015</v>
       </c>
       <c r="O127">
-        <v>76</v>
+        <v>75.75999999999999</v>
       </c>
     </row>
     <row r="128">
@@ -7261,7 +7105,7 @@
         </is>
       </c>
       <c r="H128">
-        <v>0.6666666666666572</v>
+        <v>0.7074667031563528</v>
       </c>
       <c r="I128">
         <v>2023</v>
@@ -7286,7 +7130,7 @@
         <v>2015</v>
       </c>
       <c r="O128">
-        <v>67.7</v>
+        <v>67.50045120907191</v>
       </c>
     </row>
     <row r="129">
@@ -7315,7 +7159,7 @@
         </is>
       </c>
       <c r="H129">
-        <v>1.125</v>
+        <v>1.323529411764717</v>
       </c>
       <c r="I129">
         <v>2023</v>
@@ -7340,7 +7184,7 @@
         <v>2015</v>
       </c>
       <c r="O129">
-        <v>77.2</v>
+        <v>76.95999999999999</v>
       </c>
     </row>
     <row r="130">
@@ -7369,7 +7213,7 @@
         </is>
       </c>
       <c r="H130">
-        <v>0.7187500000000036</v>
+        <v>0.7102133205520609</v>
       </c>
       <c r="I130">
         <v>2023</v>
@@ -7394,7 +7238,7 @@
         <v>2015</v>
       </c>
       <c r="O130">
-        <v>61.3</v>
+        <v>61.34427440094651</v>
       </c>
     </row>
     <row r="131">
@@ -7422,17 +7266,11 @@
           <t>MLT</t>
         </is>
       </c>
-      <c r="H131">
-        <v>0.875</v>
-      </c>
       <c r="I131">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J131">
-        <v>83.30000000000001</v>
-      </c>
-      <c r="K131">
-        <v>82.60000000000001</v>
+        <v>83.467</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -7443,12 +7281,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N131">
-        <v>2015</v>
-      </c>
-      <c r="O131">
-        <v>83.40000000000001</v>
       </c>
     </row>
     <row r="132">
@@ -7477,7 +7309,7 @@
         </is>
       </c>
       <c r="H132">
-        <v>0.6666666666666572</v>
+        <v>0.7074667031563528</v>
       </c>
       <c r="I132">
         <v>2023</v>
@@ -7502,7 +7334,7 @@
         <v>2015</v>
       </c>
       <c r="O132">
-        <v>67.7</v>
+        <v>67.50045120907191</v>
       </c>
     </row>
     <row r="133">
@@ -7531,7 +7363,7 @@
         </is>
       </c>
       <c r="H133">
-        <v>0.3125</v>
+        <v>0.3676470588235325</v>
       </c>
       <c r="I133">
         <v>2023</v>
@@ -7556,7 +7388,7 @@
         <v>2015</v>
       </c>
       <c r="O133">
-        <v>78.2</v>
+        <v>77.95999999999999</v>
       </c>
     </row>
     <row r="134">
@@ -7585,7 +7417,7 @@
         </is>
       </c>
       <c r="H134">
-        <v>1.5625</v>
+        <v>1.586110161768062</v>
       </c>
       <c r="I134">
         <v>2023</v>
@@ -7610,7 +7442,7 @@
         <v>2015</v>
       </c>
       <c r="O134">
-        <v>70.8</v>
+        <v>70.82577922077922</v>
       </c>
     </row>
     <row r="135">
@@ -7639,7 +7471,7 @@
         </is>
       </c>
       <c r="H135">
-        <v>0.875</v>
+        <v>1.029411764705891</v>
       </c>
       <c r="I135">
         <v>2023</v>
@@ -7664,7 +7496,7 @@
         <v>2015</v>
       </c>
       <c r="O135">
-        <v>79</v>
+        <v>78.76000000000001</v>
       </c>
     </row>
     <row r="136">
@@ -7693,7 +7525,7 @@
         </is>
       </c>
       <c r="H136">
-        <v>1.518750000000001</v>
+        <v>1.539306512657687</v>
       </c>
       <c r="I136">
         <v>2023</v>
@@ -7718,7 +7550,7 @@
         <v>2015</v>
       </c>
       <c r="O136">
-        <v>61.93999999999997</v>
+        <v>62.0305296515421</v>
       </c>
     </row>
     <row r="137">
@@ -7747,7 +7579,7 @@
         </is>
       </c>
       <c r="H137">
-        <v>0.8958333333333233</v>
+        <v>0.998869689087087</v>
       </c>
       <c r="I137">
         <v>2023</v>
@@ -7772,7 +7604,7 @@
         <v>2015</v>
       </c>
       <c r="O137">
-        <v>68.6666666666667</v>
+        <v>68.50207977207975</v>
       </c>
     </row>
     <row r="138">
@@ -7801,7 +7633,7 @@
         </is>
       </c>
       <c r="H138">
-        <v>0.125</v>
+        <v>0.147058823529413</v>
       </c>
       <c r="I138">
         <v>2023</v>
@@ -7826,7 +7658,7 @@
         <v>2015</v>
       </c>
       <c r="O138">
-        <v>76.3</v>
+        <v>76.06</v>
       </c>
     </row>
     <row r="139">
@@ -7855,7 +7687,7 @@
         </is>
       </c>
       <c r="H139">
-        <v>1.968749999999979</v>
+        <v>2.058220310420875</v>
       </c>
       <c r="I139">
         <v>2023</v>
@@ -7880,7 +7712,7 @@
         <v>2015</v>
       </c>
       <c r="O139">
-        <v>65.07500000000002</v>
+        <v>65.03438746424041</v>
       </c>
     </row>
     <row r="140">
@@ -7909,7 +7741,7 @@
         </is>
       </c>
       <c r="H140">
-        <v>0.875</v>
+        <v>1.029411764705891</v>
       </c>
       <c r="I140">
         <v>2023</v>
@@ -7934,7 +7766,7 @@
         <v>2015</v>
       </c>
       <c r="O140">
-        <v>76.90000000000001</v>
+        <v>76.66</v>
       </c>
     </row>
     <row r="141">
@@ -7963,7 +7795,7 @@
         </is>
       </c>
       <c r="H141">
-        <v>2.687499999999979</v>
+        <v>2.775502934194197</v>
       </c>
       <c r="I141">
         <v>2023</v>
@@ -7988,7 +7820,7 @@
         <v>2015</v>
       </c>
       <c r="O141">
-        <v>63.2</v>
+        <v>63.12773955704635</v>
       </c>
     </row>
     <row r="142">
@@ -8017,7 +7849,7 @@
         </is>
       </c>
       <c r="H142">
-        <v>1</v>
+        <v>1.176470588235304</v>
       </c>
       <c r="I142">
         <v>2023</v>
@@ -8042,7 +7874,7 @@
         <v>2015</v>
       </c>
       <c r="O142">
-        <v>78.80000000000001</v>
+        <v>78.56</v>
       </c>
     </row>
     <row r="143">
@@ -8071,7 +7903,7 @@
         </is>
       </c>
       <c r="H143">
-        <v>0.7437500000000004</v>
+        <v>0.7073297086414065</v>
       </c>
       <c r="I143">
         <v>2023</v>
@@ -8096,7 +7928,7 @@
         <v>2015</v>
       </c>
       <c r="O143">
-        <v>62.01999999999998</v>
+        <v>62.11497409598651</v>
       </c>
     </row>
     <row r="144">
@@ -8125,7 +7957,7 @@
         </is>
       </c>
       <c r="H144">
-        <v>0.6500000000000092</v>
+        <v>0.6421568627451038</v>
       </c>
       <c r="I144">
         <v>2023</v>
@@ -8150,7 +7982,7 @@
         <v>2015</v>
       </c>
       <c r="O144">
-        <v>55.90000000000001</v>
+        <v>55.9107450980392</v>
       </c>
     </row>
     <row r="145">
@@ -8179,7 +8011,7 @@
         </is>
       </c>
       <c r="H145">
-        <v>1.250000000000002</v>
+        <v>1.47058823529413</v>
       </c>
       <c r="I145">
         <v>2023</v>
@@ -8204,7 +8036,7 @@
         <v>2015</v>
       </c>
       <c r="O145">
-        <v>74.5</v>
+        <v>74.25999999999999</v>
       </c>
     </row>
     <row r="146">
@@ -8233,7 +8065,7 @@
         </is>
       </c>
       <c r="H146">
-        <v>0.4375</v>
+        <v>0.8477321289821305</v>
       </c>
       <c r="I146">
         <v>2023</v>
@@ -8258,7 +8090,7 @@
         <v>2015</v>
       </c>
       <c r="O146">
-        <v>82.85000000000001</v>
+        <v>82.28527000777002</v>
       </c>
     </row>
     <row r="147">
@@ -8286,17 +8118,11 @@
           <t>NOR</t>
         </is>
       </c>
-      <c r="H147">
-        <v>1.0625</v>
-      </c>
       <c r="I147">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J147">
-        <v>83.30000000000001</v>
-      </c>
-      <c r="K147">
-        <v>82.30000000000001</v>
+        <v>83.45999999999999</v>
       </c>
       <c r="L147" t="inlineStr">
         <is>
@@ -8307,12 +8133,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N147">
-        <v>2015</v>
-      </c>
-      <c r="O147">
-        <v>83.25</v>
       </c>
     </row>
     <row r="148">
@@ -8341,7 +8161,7 @@
         </is>
       </c>
       <c r="H148">
-        <v>1.708333333333329</v>
+        <v>1.690624411820075</v>
       </c>
       <c r="I148">
         <v>2023</v>
@@ -8366,7 +8186,7 @@
         <v>2015</v>
       </c>
       <c r="O148">
-        <v>69.26666666666669</v>
+        <v>69.26307246376813</v>
       </c>
     </row>
     <row r="149">
@@ -8395,7 +8215,7 @@
         </is>
       </c>
       <c r="H149">
-        <v>0.375</v>
+        <v>0.3807324067673896</v>
       </c>
       <c r="I149">
         <v>2023</v>
@@ -8420,7 +8240,7 @@
         <v>2015</v>
       </c>
       <c r="O149">
-        <v>64.02499999999999</v>
+        <v>63.87965181936301</v>
       </c>
     </row>
     <row r="150">
@@ -8449,7 +8269,7 @@
         </is>
       </c>
       <c r="H150">
-        <v>0.3125</v>
+        <v>0.5953282828282838</v>
       </c>
       <c r="I150">
         <v>2023</v>
@@ -8474,7 +8294,7 @@
         <v>2015</v>
       </c>
       <c r="O150">
-        <v>82.90000000000001</v>
+        <v>82.33352813852815</v>
       </c>
     </row>
     <row r="151">
@@ -8503,7 +8323,7 @@
         </is>
       </c>
       <c r="H151">
-        <v>0.4375</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I151">
         <v>2023</v>
@@ -8528,7 +8348,7 @@
         <v>2015</v>
       </c>
       <c r="O151">
-        <v>80.90000000000001</v>
+        <v>80.65058823529414</v>
       </c>
     </row>
     <row r="152">
@@ -8557,7 +8377,7 @@
         </is>
       </c>
       <c r="H152">
-        <v>0.8333333333333215</v>
+        <v>0.9247743954640502</v>
       </c>
       <c r="I152">
         <v>2023</v>
@@ -8582,7 +8402,7 @@
         <v>2015</v>
       </c>
       <c r="O152">
-        <v>68</v>
+        <v>67.75045120907191</v>
       </c>
     </row>
     <row r="153">
@@ -8611,7 +8431,7 @@
         </is>
       </c>
       <c r="H153">
-        <v>1.25</v>
+        <v>1.47058823529413</v>
       </c>
       <c r="I153">
         <v>2023</v>
@@ -8636,7 +8456,7 @@
         <v>2015</v>
       </c>
       <c r="O153">
-        <v>79.2</v>
+        <v>78.95999999999999</v>
       </c>
     </row>
     <row r="154">
@@ -8665,7 +8485,7 @@
         </is>
       </c>
       <c r="H154">
-        <v>1.25</v>
+        <v>1.47058823529413</v>
       </c>
       <c r="I154">
         <v>2023</v>
@@ -8690,7 +8510,7 @@
         <v>2015</v>
       </c>
       <c r="O154">
-        <v>77.30000000000001</v>
+        <v>77.06</v>
       </c>
     </row>
     <row r="155">
@@ -8719,7 +8539,7 @@
         </is>
       </c>
       <c r="H155">
-        <v>0.25</v>
+        <v>0.2380952380952408</v>
       </c>
       <c r="I155">
         <v>2023</v>
@@ -8744,7 +8564,7 @@
         <v>2015</v>
       </c>
       <c r="O155">
-        <v>71</v>
+        <v>71.00261904761905</v>
       </c>
     </row>
     <row r="156">
@@ -8773,7 +8593,7 @@
         </is>
       </c>
       <c r="H156">
-        <v>0.125</v>
+        <v>0.1136363636363633</v>
       </c>
       <c r="I156">
         <v>2023</v>
@@ -8798,7 +8618,7 @@
         <v>2015</v>
       </c>
       <c r="O156">
-        <v>70.7</v>
+        <v>70.73941558441558</v>
       </c>
     </row>
     <row r="157">
@@ -8827,7 +8647,7 @@
         </is>
       </c>
       <c r="H157">
-        <v>0.6666666666666572</v>
+        <v>0.6622011394936145</v>
       </c>
       <c r="I157">
         <v>2023</v>
@@ -8852,7 +8672,7 @@
         <v>2015</v>
       </c>
       <c r="O157">
-        <v>66.90000000000001</v>
+        <v>66.84035982440808</v>
       </c>
     </row>
     <row r="158">
@@ -8881,7 +8701,7 @@
         </is>
       </c>
       <c r="H158">
-        <v>0.625</v>
+        <v>0.7352941176470651</v>
       </c>
       <c r="I158">
         <v>2023</v>
@@ -8906,7 +8726,7 @@
         <v>2015</v>
       </c>
       <c r="O158">
-        <v>79.2</v>
+        <v>78.95999999999999</v>
       </c>
     </row>
     <row r="159">
@@ -8935,7 +8755,7 @@
         </is>
       </c>
       <c r="H159">
-        <v>0.625</v>
+        <v>0.8812957875457883</v>
       </c>
       <c r="I159">
         <v>2023</v>
@@ -8960,7 +8780,7 @@
         <v>2015</v>
       </c>
       <c r="O159">
-        <v>82.30000000000001</v>
+        <v>81.80445970695972</v>
       </c>
     </row>
     <row r="160">
@@ -8989,7 +8809,7 @@
         </is>
       </c>
       <c r="H160">
-        <v>0.5000000000000018</v>
+        <v>0.5882352941176521</v>
       </c>
       <c r="I160">
         <v>2023</v>
@@ -9014,7 +8834,7 @@
         <v>2015</v>
       </c>
       <c r="O160">
-        <v>74.40000000000001</v>
+        <v>74.16</v>
       </c>
     </row>
     <row r="161">
@@ -9043,7 +8863,7 @@
         </is>
       </c>
       <c r="H161">
-        <v>0.6875</v>
+        <v>1.420076451326452</v>
       </c>
       <c r="I161">
         <v>2023</v>
@@ -9068,7 +8888,7 @@
         <v>2015</v>
       </c>
       <c r="O161">
-        <v>82.75</v>
+        <v>82.17877011877012</v>
       </c>
     </row>
     <row r="162">
@@ -9097,7 +8917,7 @@
         </is>
       </c>
       <c r="H162">
-        <v>0.1875</v>
+        <v>0.2205882352941195</v>
       </c>
       <c r="I162">
         <v>2023</v>
@@ -9122,7 +8942,7 @@
         <v>2015</v>
       </c>
       <c r="O162">
-        <v>75.10000000000001</v>
+        <v>74.86</v>
       </c>
     </row>
     <row r="163">
@@ -9151,7 +8971,7 @@
         </is>
       </c>
       <c r="H163">
-        <v>-5.249999999999984</v>
+        <v>-5.637302832051938</v>
       </c>
       <c r="I163">
         <v>2023</v>
@@ -9176,7 +8996,7 @@
         <v>2015</v>
       </c>
       <c r="O163">
-        <v>76.2</v>
+        <v>75.95999999999999</v>
       </c>
     </row>
     <row r="164">
@@ -9204,17 +9024,11 @@
           <t>PYF</t>
         </is>
       </c>
-      <c r="H164">
-        <v>2.0625</v>
-      </c>
       <c r="I164">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J164">
-        <v>84.10000000000001</v>
-      </c>
-      <c r="K164">
-        <v>82.30000000000001</v>
+        <v>84.19199999999999</v>
       </c>
       <c r="L164" t="inlineStr">
         <is>
@@ -9225,12 +9039,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N164">
-        <v>2015</v>
-      </c>
-      <c r="O164">
-        <v>83.25</v>
       </c>
     </row>
     <row r="165">
@@ -9259,7 +9067,7 @@
         </is>
       </c>
       <c r="H165">
-        <v>0.375</v>
+        <v>0.9206800144300118</v>
       </c>
       <c r="I165">
         <v>2023</v>
@@ -9284,7 +9092,7 @@
         <v>2015</v>
       </c>
       <c r="O165">
-        <v>83</v>
+        <v>82.431727994228</v>
       </c>
     </row>
     <row r="166">
@@ -9313,7 +9121,7 @@
         </is>
       </c>
       <c r="H166">
-        <v>0.75</v>
+        <v>0.8823529411764781</v>
       </c>
       <c r="I166">
         <v>2023</v>
@@ -9338,7 +9146,7 @@
         <v>2015</v>
       </c>
       <c r="O166">
-        <v>76.3</v>
+        <v>76.06</v>
       </c>
     </row>
     <row r="167">
@@ -9367,7 +9175,7 @@
         </is>
       </c>
       <c r="H167">
-        <v>1.1875</v>
+        <v>1.340299277605785</v>
       </c>
       <c r="I167">
         <v>2023</v>
@@ -9392,7 +9200,7 @@
         <v>2015</v>
       </c>
       <c r="O167">
-        <v>72.90000000000001</v>
+        <v>72.73719298245614</v>
       </c>
     </row>
     <row r="168">
@@ -9421,7 +9229,7 @@
         </is>
       </c>
       <c r="H168">
-        <v>0.9999999999999858</v>
+        <v>1.108107728797384</v>
       </c>
       <c r="I168">
         <v>2023</v>
@@ -9446,7 +9254,7 @@
         <v>2015</v>
       </c>
       <c r="O168">
-        <v>67.8</v>
+        <v>67.58378454240527</v>
       </c>
     </row>
     <row r="169">
@@ -9475,7 +9283,7 @@
         </is>
       </c>
       <c r="H169">
-        <v>0.5625</v>
+        <v>0.6617647058823586</v>
       </c>
       <c r="I169">
         <v>2023</v>
@@ -9500,7 +9308,7 @@
         <v>2015</v>
       </c>
       <c r="O169">
-        <v>79.40000000000001</v>
+        <v>79.16</v>
       </c>
     </row>
     <row r="170">
@@ -9529,7 +9337,7 @@
         </is>
       </c>
       <c r="H170">
-        <v>0.7916666666666554</v>
+        <v>0.7905493537793298</v>
       </c>
       <c r="I170">
         <v>2023</v>
@@ -9554,7 +9362,7 @@
         <v>2015</v>
       </c>
       <c r="O170">
-        <v>66.8</v>
+        <v>66.75598482440807</v>
       </c>
     </row>
     <row r="171">
@@ -9583,7 +9391,7 @@
         </is>
       </c>
       <c r="H171">
-        <v>1.020833333333323</v>
+        <v>1.107565341261001</v>
       </c>
       <c r="I171">
         <v>2023</v>
@@ -9608,7 +9416,7 @@
         <v>2015</v>
       </c>
       <c r="O171">
-        <v>68.6666666666667</v>
+        <v>68.50207977207975</v>
       </c>
     </row>
     <row r="172">
@@ -9636,17 +9444,11 @@
           <t>SGP</t>
         </is>
       </c>
-      <c r="H172">
-        <v>1.25</v>
-      </c>
       <c r="I172">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J172">
-        <v>83.7</v>
-      </c>
-      <c r="K172">
-        <v>82.7</v>
+        <v>83.863</v>
       </c>
       <c r="L172" t="inlineStr">
         <is>
@@ -9657,12 +9459,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N172">
-        <v>2015</v>
-      </c>
-      <c r="O172">
-        <v>83.5</v>
       </c>
     </row>
     <row r="173">
@@ -9691,7 +9487,7 @@
         </is>
       </c>
       <c r="H173">
-        <v>0.75</v>
+        <v>0.7321428571428612</v>
       </c>
       <c r="I173">
         <v>2023</v>
@@ -9716,7 +9512,7 @@
         <v>2015</v>
       </c>
       <c r="O173">
-        <v>70.90000000000001</v>
+        <v>70.91214285714285</v>
       </c>
     </row>
     <row r="174">
@@ -9745,7 +9541,7 @@
         </is>
       </c>
       <c r="H174">
-        <v>1.756250000000012</v>
+        <v>1.774990146176792</v>
       </c>
       <c r="I174">
         <v>2023</v>
@@ -9770,7 +9566,7 @@
         <v>2015</v>
       </c>
       <c r="O174">
-        <v>59.37999999999993</v>
+        <v>59.2325190205592</v>
       </c>
     </row>
     <row r="175">
@@ -9799,7 +9595,7 @@
         </is>
       </c>
       <c r="H175">
-        <v>0.6875</v>
+        <v>0.749269005847955</v>
       </c>
       <c r="I175">
         <v>2023</v>
@@ -9824,7 +9620,7 @@
         <v>2015</v>
       </c>
       <c r="O175">
-        <v>72.60000000000001</v>
+        <v>72.46105263157895</v>
       </c>
     </row>
     <row r="176">
@@ -9852,17 +9648,11 @@
           <t>SMR</t>
         </is>
       </c>
-      <c r="H176">
-        <v>1.375</v>
-      </c>
       <c r="I176">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J176">
-        <v>85.7</v>
-      </c>
-      <c r="K176">
-        <v>84.60000000000001</v>
+        <v>85.81699999999999</v>
       </c>
       <c r="L176" t="inlineStr">
         <is>
@@ -9873,12 +9663,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N176">
-        <v>2015</v>
-      </c>
-      <c r="O176">
-        <v>85.40000000000001</v>
       </c>
     </row>
     <row r="177">
@@ -9907,7 +9691,7 @@
         </is>
       </c>
       <c r="H177">
-        <v>0.9250000000000131</v>
+        <v>0.979797407708066</v>
       </c>
       <c r="I177">
         <v>2023</v>
@@ -9932,7 +9716,7 @@
         <v>2015</v>
       </c>
       <c r="O177">
-        <v>59.05999999999995</v>
+        <v>58.87272933225095</v>
       </c>
     </row>
     <row r="178">
@@ -9961,7 +9745,7 @@
         </is>
       </c>
       <c r="H178">
-        <v>0.6875</v>
+        <v>0.8088235294117716</v>
       </c>
       <c r="I178">
         <v>2023</v>
@@ -9986,7 +9770,7 @@
         <v>2015</v>
       </c>
       <c r="O178">
-        <v>77.30000000000001</v>
+        <v>77.06</v>
       </c>
     </row>
     <row r="179">
@@ -10015,7 +9799,7 @@
         </is>
       </c>
       <c r="H179">
-        <v>4.656250000000052</v>
+        <v>4.642704248409249</v>
       </c>
       <c r="I179">
         <v>2023</v>
@@ -10040,7 +9824,7 @@
         <v>2015</v>
       </c>
       <c r="O179">
-        <v>43</v>
+        <v>43.24333669733558</v>
       </c>
     </row>
     <row r="180">
@@ -10069,7 +9853,7 @@
         </is>
       </c>
       <c r="H180">
-        <v>1.854166666666654</v>
+        <v>1.911437395133058</v>
       </c>
       <c r="I180">
         <v>2023</v>
@@ -10094,7 +9878,7 @@
         <v>2015</v>
       </c>
       <c r="O180">
-        <v>68.33333333333334</v>
+        <v>68.08346764346763</v>
       </c>
     </row>
     <row r="181">
@@ -10123,7 +9907,7 @@
         </is>
       </c>
       <c r="H181">
-        <v>1.875000000000002</v>
+        <v>2.094943240454086</v>
       </c>
       <c r="I181">
         <v>2023</v>
@@ -10148,7 +9932,7 @@
         <v>2015</v>
       </c>
       <c r="O181">
-        <v>72.2</v>
+        <v>72.08210526315791</v>
       </c>
     </row>
     <row r="182">
@@ -10177,7 +9961,7 @@
         </is>
       </c>
       <c r="H182">
-        <v>1.0625</v>
+        <v>1.250000000000011</v>
       </c>
       <c r="I182">
         <v>2023</v>
@@ -10202,7 +9986,7 @@
         <v>2015</v>
       </c>
       <c r="O182">
-        <v>78.2</v>
+        <v>77.95999999999999</v>
       </c>
     </row>
     <row r="183">
@@ -10231,7 +10015,7 @@
         </is>
       </c>
       <c r="H183">
-        <v>0.6875</v>
+        <v>0.9333791208791204</v>
       </c>
       <c r="I183">
         <v>2023</v>
@@ -10256,7 +10040,7 @@
         <v>2015</v>
       </c>
       <c r="O183">
-        <v>82.10000000000001</v>
+        <v>81.66395604395605</v>
       </c>
     </row>
     <row r="184">
@@ -10284,17 +10068,11 @@
           <t>SWE</t>
         </is>
       </c>
-      <c r="H184">
-        <v>1.125</v>
-      </c>
       <c r="I184">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="J184">
-        <v>83.30000000000001</v>
-      </c>
-      <c r="K184">
-        <v>82.2</v>
+        <v>83.42400000000001</v>
       </c>
       <c r="L184" t="inlineStr">
         <is>
@@ -10305,12 +10083,6 @@
         <is>
           <t>Life expectancy at birth, total (years)</t>
         </is>
-      </c>
-      <c r="N184">
-        <v>2015</v>
-      </c>
-      <c r="O184">
-        <v>83.2</v>
       </c>
     </row>
     <row r="185">
@@ -10339,7 +10111,7 @@
         </is>
       </c>
       <c r="H185">
-        <v>2.656250000000012</v>
+        <v>2.727284162159439</v>
       </c>
       <c r="I185">
         <v>2023</v>
@@ -10364,7 +10136,7 @@
         <v>2015</v>
       </c>
       <c r="O185">
-        <v>58.90000000000001</v>
+        <v>58.68905586286319</v>
       </c>
     </row>
     <row r="186">
@@ -10393,7 +10165,7 @@
         </is>
       </c>
       <c r="H186">
-        <v>0.3125</v>
+        <v>0.3676470588235325</v>
       </c>
       <c r="I186">
         <v>2023</v>
@@ -10418,7 +10190,7 @@
         <v>2015</v>
       </c>
       <c r="O186">
-        <v>77.5</v>
+        <v>77.26000000000001</v>
       </c>
     </row>
     <row r="187">
@@ -10447,7 +10219,7 @@
         </is>
       </c>
       <c r="H187">
-        <v>0.375</v>
+        <v>0.4289215686274535</v>
       </c>
       <c r="I187">
         <v>2023</v>
@@ -10472,7 +10244,7 @@
         <v>2015</v>
       </c>
       <c r="O187">
-        <v>73.90000000000001</v>
+        <v>73.67666666666666</v>
       </c>
     </row>
     <row r="188">
@@ -10501,7 +10273,7 @@
         </is>
       </c>
       <c r="H188">
-        <v>4.427083333333307</v>
+        <v>4.542749529303654</v>
       </c>
       <c r="I188">
         <v>2023</v>
@@ -10526,7 +10298,7 @@
         <v>2015</v>
       </c>
       <c r="O188">
-        <v>65.82500000000003</v>
+        <v>65.85537673427143</v>
       </c>
     </row>
     <row r="189">
@@ -10555,7 +10327,7 @@
         </is>
       </c>
       <c r="H189">
-        <v>0.4375</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I189">
         <v>2023</v>
@@ -10580,7 +10352,7 @@
         <v>2015</v>
       </c>
       <c r="O189">
-        <v>78.90000000000001</v>
+        <v>78.66</v>
       </c>
     </row>
     <row r="190">
@@ -10609,7 +10381,7 @@
         </is>
       </c>
       <c r="H190">
-        <v>0.9500000000000135</v>
+        <v>0.9402360944377808</v>
       </c>
       <c r="I190">
         <v>2023</v>
@@ -10634,7 +10406,7 @@
         <v>2015</v>
       </c>
       <c r="O190">
-        <v>55.3</v>
+        <v>55.33427450980393</v>
       </c>
     </row>
     <row r="191">
@@ -10663,7 +10435,7 @@
         </is>
       </c>
       <c r="H191">
-        <v>1.09375</v>
+        <v>1.082993868845039</v>
       </c>
       <c r="I191">
         <v>2023</v>
@@ -10688,7 +10460,7 @@
         <v>2015</v>
       </c>
       <c r="O191">
-        <v>62.40000000000001</v>
+        <v>62.45433814821867</v>
       </c>
     </row>
     <row r="192">
@@ -10717,7 +10489,7 @@
         </is>
       </c>
       <c r="H192">
-        <v>-0.125</v>
+        <v>-0.147058823529413</v>
       </c>
       <c r="I192">
         <v>2023</v>
@@ -10742,7 +10514,7 @@
         <v>2015</v>
       </c>
       <c r="O192">
-        <v>78.2</v>
+        <v>77.95999999999999</v>
       </c>
     </row>
     <row r="193">
@@ -10771,7 +10543,7 @@
         </is>
       </c>
       <c r="H193">
-        <v>1.3125</v>
+        <v>1.360641186299084</v>
       </c>
       <c r="I193">
         <v>2023</v>
@@ -10796,7 +10568,7 @@
         <v>2015</v>
       </c>
       <c r="O193">
-        <v>71.3</v>
+        <v>71.27404761904761</v>
       </c>
     </row>
     <row r="194">
@@ -10825,7 +10597,7 @@
         </is>
       </c>
       <c r="H194">
-        <v>0.625</v>
+        <v>0.5957792207792245</v>
       </c>
       <c r="I194">
         <v>2023</v>
@@ -10850,7 +10622,7 @@
         <v>2015</v>
       </c>
       <c r="O194">
-        <v>70.7</v>
+        <v>70.73941558441558</v>
       </c>
     </row>
     <row r="195">
@@ -10879,7 +10651,7 @@
         </is>
       </c>
       <c r="H195">
-        <v>0.9999999999999858</v>
+        <v>1.099774395464049</v>
       </c>
       <c r="I195">
         <v>2023</v>
@@ -10904,7 +10676,7 @@
         <v>2015</v>
       </c>
       <c r="O195">
-        <v>67.7</v>
+        <v>67.50045120907191</v>
       </c>
     </row>
     <row r="196">
@@ -10933,7 +10705,7 @@
         </is>
       </c>
       <c r="H196">
-        <v>0.625</v>
+        <v>0.706699346405232</v>
       </c>
       <c r="I196">
         <v>2023</v>
@@ -10958,7 +10730,7 @@
         <v>2015</v>
       </c>
       <c r="O196">
-        <v>73.5</v>
+        <v>73.29888888888887</v>
       </c>
     </row>
     <row r="197">
@@ -10987,7 +10759,7 @@
         </is>
       </c>
       <c r="H197">
-        <v>0.3750000000000018</v>
+        <v>0.4411764705882391</v>
       </c>
       <c r="I197">
         <v>2023</v>
@@ -11012,7 +10784,7 @@
         <v>2015</v>
       </c>
       <c r="O197">
-        <v>74.5</v>
+        <v>74.25999999999999</v>
       </c>
     </row>
     <row r="198">
@@ -11041,7 +10813,7 @@
         </is>
       </c>
       <c r="H198">
-        <v>1</v>
+        <v>1.176470588235304</v>
       </c>
       <c r="I198">
         <v>2023</v>
@@ -11066,7 +10838,7 @@
         <v>2015</v>
       </c>
       <c r="O198">
-        <v>76.5</v>
+        <v>76.25999999999999</v>
       </c>
     </row>
     <row r="199">
@@ -11095,7 +10867,7 @@
         </is>
       </c>
       <c r="H199">
-        <v>0.4375</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I199">
         <v>2023</v>
@@ -11120,7 +10892,7 @@
         <v>2015</v>
       </c>
       <c r="O199">
-        <v>78.10000000000001</v>
+        <v>77.86</v>
       </c>
     </row>
     <row r="200">
@@ -11149,7 +10921,7 @@
         </is>
       </c>
       <c r="H200">
-        <v>0.7083333333333233</v>
+        <v>0.7619538826435335</v>
       </c>
       <c r="I200">
         <v>2023</v>
@@ -11174,7 +10946,7 @@
         <v>2015</v>
       </c>
       <c r="O200">
-        <v>67.8</v>
+        <v>67.58378454240527</v>
       </c>
     </row>
     <row r="201">
@@ -11203,7 +10975,7 @@
         </is>
       </c>
       <c r="H201">
-        <v>0.4375</v>
+        <v>0.5193014705882391</v>
       </c>
       <c r="I201">
         <v>2023</v>
@@ -11228,7 +11000,7 @@
         <v>2015</v>
       </c>
       <c r="O201">
-        <v>81.5</v>
+        <v>81.19558823529412</v>
       </c>
     </row>
     <row r="202">
@@ -11257,7 +11029,7 @@
         </is>
       </c>
       <c r="H202">
-        <v>1.291666666666648</v>
+        <v>1.303030472878092</v>
       </c>
       <c r="I202">
         <v>2023</v>
@@ -11282,7 +11054,7 @@
         <v>2015</v>
       </c>
       <c r="O202">
-        <v>66.3</v>
+        <v>66.3474225669639</v>
       </c>
     </row>
     <row r="203">
@@ -11311,7 +11083,7 @@
         </is>
       </c>
       <c r="H203">
-        <v>1.895833333333307</v>
+        <v>1.996707107411511</v>
       </c>
       <c r="I203">
         <v>2023</v>
@@ -11336,7 +11108,7 @@
         <v>2015</v>
       </c>
       <c r="O203">
-        <v>66.2</v>
+        <v>66.26506962578742</v>
       </c>
     </row>
     <row r="204">
@@ -11365,7 +11137,7 @@
         </is>
       </c>
       <c r="H204">
-        <v>0.4375</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I204">
         <v>2023</v>
@@ -11390,7 +11162,7 @@
         <v>2015</v>
       </c>
       <c r="O204">
-        <v>74.3</v>
+        <v>74.06</v>
       </c>
     </row>
     <row r="205">
@@ -11419,7 +11191,7 @@
         </is>
       </c>
       <c r="H205">
-        <v>0.5</v>
+        <v>0.5882352941176521</v>
       </c>
       <c r="I205">
         <v>2023</v>
@@ -11444,7 +11216,7 @@
         <v>2015</v>
       </c>
       <c r="O205">
-        <v>78.90000000000001</v>
+        <v>78.66</v>
       </c>
     </row>
     <row r="206">
@@ -11473,7 +11245,7 @@
         </is>
       </c>
       <c r="H206">
-        <v>0.375</v>
+        <v>0.4411764705882391</v>
       </c>
       <c r="I206">
         <v>2023</v>
@@ -11498,7 +11270,7 @@
         <v>2015</v>
       </c>
       <c r="O206">
-        <v>80.30000000000001</v>
+        <v>80.06</v>
       </c>
     </row>
     <row r="207">
@@ -11527,7 +11299,7 @@
         </is>
       </c>
       <c r="H207">
-        <v>0.6875</v>
+        <v>0.760233918128657</v>
       </c>
       <c r="I207">
         <v>2023</v>
@@ -11552,7 +11324,7 @@
         <v>2015</v>
       </c>
       <c r="O207">
-        <v>72.90000000000001</v>
+        <v>72.73719298245614</v>
       </c>
     </row>
     <row r="208">
@@ -11581,7 +11353,7 @@
         </is>
       </c>
       <c r="H208">
-        <v>0.4375</v>
+        <v>0.4572368421052637</v>
       </c>
       <c r="I208">
         <v>2023</v>
@@ -11606,7 +11378,7 @@
         <v>2015</v>
       </c>
       <c r="O208">
-        <v>72.10000000000001</v>
+        <v>71.99210526315788</v>
       </c>
     </row>
     <row r="209">
@@ -11635,7 +11407,7 @@
         </is>
       </c>
       <c r="H209">
-        <v>-0.3125</v>
+        <v>-0.3635620915032707</v>
       </c>
       <c r="I209">
         <v>2023</v>
@@ -11660,7 +11432,7 @@
         <v>2015</v>
       </c>
       <c r="O209">
-        <v>74.60000000000001</v>
+        <v>74.36</v>
       </c>
     </row>
     <row r="210">
@@ -11689,7 +11461,7 @@
         </is>
       </c>
       <c r="H210">
-        <v>0.4375</v>
+        <v>0.5147058823529456</v>
       </c>
       <c r="I210">
         <v>2023</v>
@@ -11714,7 +11486,7 @@
         <v>2015</v>
       </c>
       <c r="O210">
-        <v>78.2</v>
+        <v>77.95999999999999</v>
       </c>
     </row>
     <row r="211">
@@ -11743,7 +11515,7 @@
         </is>
       </c>
       <c r="H211">
-        <v>0.75</v>
+        <v>0.8823529411764781</v>
       </c>
       <c r="I211">
         <v>2023</v>
@@ -11768,7 +11540,7 @@
         <v>2015</v>
       </c>
       <c r="O211">
-        <v>75.90000000000001</v>
+        <v>75.66</v>
       </c>
     </row>
     <row r="212">
@@ -11797,7 +11569,7 @@
         </is>
       </c>
       <c r="H212">
-        <v>0.375</v>
+        <v>0.4411764705882391</v>
       </c>
       <c r="I212">
         <v>2023</v>
@@ -11822,7 +11594,7 @@
         <v>2015</v>
       </c>
       <c r="O212">
-        <v>75.60000000000001</v>
+        <v>75.36</v>
       </c>
     </row>
     <row r="213">
@@ -11851,7 +11623,7 @@
         </is>
       </c>
       <c r="H213">
-        <v>0.8125</v>
+        <v>0.8457602339181296</v>
       </c>
       <c r="I213">
         <v>2023</v>
@@ -11876,7 +11648,7 @@
         <v>2015</v>
       </c>
       <c r="O213">
-        <v>71.8</v>
+        <v>71.7221052631579</v>
       </c>
     </row>
     <row r="214">
@@ -11905,7 +11677,7 @@
         </is>
       </c>
       <c r="H214">
-        <v>0.375</v>
+        <v>0.4057017543859658</v>
       </c>
       <c r="I214">
         <v>2023</v>
@@ -11930,7 +11702,7 @@
         <v>2015</v>
       </c>
       <c r="O214">
-        <v>72.7</v>
+        <v>72.55578947368421</v>
       </c>
     </row>
     <row r="215">
@@ -11959,7 +11731,7 @@
         </is>
       </c>
       <c r="H215">
-        <v>1.25</v>
+        <v>1.47058823529413</v>
       </c>
       <c r="I215">
         <v>2023</v>
@@ -11984,7 +11756,7 @@
         <v>2015</v>
       </c>
       <c r="O215">
-        <v>77.60000000000001</v>
+        <v>77.36</v>
       </c>
     </row>
     <row r="216">
@@ -12013,7 +11785,7 @@
         </is>
       </c>
       <c r="H216">
-        <v>1.270833333333325</v>
+        <v>1.309585543281203</v>
       </c>
       <c r="I216">
         <v>2023</v>
@@ -12038,7 +11810,7 @@
         <v>2015</v>
       </c>
       <c r="O216">
-        <v>68.8666666666667</v>
+        <v>68.75512944382508</v>
       </c>
     </row>
     <row r="217">
@@ -12067,7 +11839,7 @@
         </is>
       </c>
       <c r="H217">
-        <v>0.8333333333333215</v>
+        <v>0.814900003129976</v>
       </c>
       <c r="I217">
         <v>2023</v>
@@ -12092,7 +11864,7 @@
         <v>2015</v>
       </c>
       <c r="O217">
-        <v>66.5</v>
+        <v>66.51053027895352</v>
       </c>
     </row>
     <row r="218">
@@ -12121,7 +11893,7 @@
         </is>
       </c>
       <c r="H218">
-        <v>2.010416666666652</v>
+        <v>2.047285769696542</v>
       </c>
       <c r="I218">
         <v>2023</v>
@@ -12146,7 +11918,7 @@
         <v>2015</v>
       </c>
       <c r="O218">
-        <v>63.87500000000002</v>
+        <v>63.71379816082639</v>
       </c>
     </row>
     <row r="219">
@@ -12175,7 +11947,7 @@
         </is>
       </c>
       <c r="H219">
-        <v>1.1875</v>
+        <v>1.173595834447006</v>
       </c>
       <c r="I219">
         <v>2023</v>
@@ -12200,7 +11972,7 @@
         <v>2015</v>
       </c>
       <c r="O219">
-        <v>62.2</v>
+        <v>62.28578217679464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>